<commit_message>
Updated test report revision history
Signed-off-by: Prasad Jondhale <prasad.jondhale@ti.com>
</commit_message>
<xml_diff>
--- a/docs/test_report/ethfw_testreport.xlsx
+++ b/docs/test_report/ethfw_testreport.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="0" windowWidth="12300" windowHeight="2610" tabRatio="599" activeTab="1"/>
+    <workbookView xWindow="-15" yWindow="0" windowWidth="12300" windowHeight="2610" tabRatio="599" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="176">
   <si>
     <t>Test is not required for this release (e.g., test case not supported for targeted platform)</t>
   </si>
@@ -552,6 +552,15 @@
   </si>
   <si>
     <t>EthFw_J7_00.08.00_EA8</t>
+  </si>
+  <si>
+    <t>Prasad Jondhale</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Downloaded from FoQus for 0.8 release and updated the summary tab and test details</t>
   </si>
 </sst>
 </file>
@@ -1330,19 +1339,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="9">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
     <xf numFmtId="9" fontId="12" fillId="2" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="41"/>
     <xf numFmtId="9" fontId="12" fillId="2" borderId="41"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="41"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="41"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="41"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="41"/>
   </cellStyleXfs>
   <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="6" fillId="2" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1500,15 +1515,6 @@
     <xf numFmtId="15" fontId="0" fillId="2" borderId="50" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="2" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1533,12 +1539,36 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1560,6 +1590,39 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="42" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="31" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="43" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1569,6 +1632,36 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="40" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="41" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1590,24 +1683,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1617,57 +1698,6 @@
     <xf numFmtId="0" fontId="9" fillId="13" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="40" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="41" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="42" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="31" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="43" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1682,35 +1712,8 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="48" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="49" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="11">
-    <cellStyle name="Normal" xfId="6"/>
-    <cellStyle name="Normal" xfId="7"/>
-    <cellStyle name="Normal" xfId="8"/>
+  <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2"/>
     <cellStyle name="Normal 2 2" xfId="5"/>
@@ -2131,30 +2134,30 @@
   <dimension ref="A1:I18"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="15" style="4" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
       <c r="I2" s="59"/>
     </row>
     <row r="3" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
+      <c r="A3" s="6"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="63" t="s">
@@ -2168,148 +2171,148 @@
       <c r="G4" s="65"/>
     </row>
     <row r="5" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="66" t="s">
         <v>170</v>
       </c>
-      <c r="C5" s="118"/>
-      <c r="D5" s="118"/>
-      <c r="E5" s="118"/>
-      <c r="F5" s="118"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="67"/>
+      <c r="F5" s="67"/>
       <c r="G5" s="68"/>
     </row>
-    <row r="6" spans="1:9" s="5" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:9" s="8" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B6" s="119" t="s">
+      <c r="B6" s="69" t="s">
         <v>172</v>
       </c>
-      <c r="C6" s="120"/>
-      <c r="D6" s="120"/>
-      <c r="E6" s="120"/>
-      <c r="F6" s="120"/>
-      <c r="G6" s="121"/>
-    </row>
-    <row r="7" spans="1:9" s="1" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="C6" s="70"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="70"/>
+      <c r="F6" s="70"/>
+      <c r="G6" s="71"/>
+    </row>
+    <row r="7" spans="1:9" s="4" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="125">
+      <c r="B7" s="72">
         <v>43557</v>
       </c>
-      <c r="C7" s="120"/>
-      <c r="D7" s="120"/>
-      <c r="E7" s="120"/>
-      <c r="F7" s="120"/>
-      <c r="G7" s="121"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-    </row>
-    <row r="8" spans="1:9" s="1" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="C7" s="70"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+    </row>
+    <row r="8" spans="1:9" s="4" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="122" t="s">
+      <c r="B8" s="73" t="s">
         <v>171</v>
       </c>
-      <c r="C8" s="123"/>
-      <c r="D8" s="123"/>
-      <c r="E8" s="123"/>
-      <c r="F8" s="123"/>
-      <c r="G8" s="124"/>
-    </row>
-    <row r="9" spans="1:9" s="1" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="C8" s="74"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="G8" s="75"/>
+    </row>
+    <row r="9" spans="1:9" s="4" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="66" t="s">
         <v>103</v>
       </c>
-      <c r="C9" s="67"/>
-      <c r="D9" s="67"/>
-      <c r="E9" s="67"/>
-      <c r="F9" s="67"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+      <c r="F9" s="76"/>
       <c r="G9" s="68"/>
     </row>
-    <row r="10" spans="1:9" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6"/>
+    </row>
+    <row r="11" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:9" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="60" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="61"/>
       <c r="C12" s="62"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-    </row>
-    <row r="13" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+    </row>
+    <row r="13" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="56" t="s">
+      <c r="B13" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C13" s="56"/>
-    </row>
-    <row r="14" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
+      <c r="C13" s="1"/>
+    </row>
+    <row r="14" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="12">
         <v>9</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="8" t="s">
+    <row r="15" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="12">
         <v>0</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="12" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
+    <row r="16" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="12">
         <v>0</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="12" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="17" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="8" t="s">
+    <row r="17" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="12">
         <v>0</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="12" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="18" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
+    <row r="18" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="12">
         <v>0</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="12" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2336,721 +2339,721 @@
   <dimension ref="A1:AH14"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="51.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="60.7109375" style="10" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" style="10" customWidth="1"/>
-    <col min="6" max="6" width="34.42578125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="30.42578125" style="10" customWidth="1"/>
-    <col min="8" max="9" width="19.28515625" style="10" customWidth="1"/>
-    <col min="10" max="23" width="4.7109375" style="10" customWidth="1"/>
-    <col min="24" max="24" width="19.28515625" style="10" customWidth="1"/>
-    <col min="25" max="27" width="4.7109375" style="10" customWidth="1"/>
-    <col min="28" max="28" width="19.28515625" style="10" customWidth="1"/>
-    <col min="29" max="29" width="16.42578125" style="10" customWidth="1"/>
-    <col min="30" max="30" width="13.42578125" style="5" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="14.28515625" style="10" hidden="1" customWidth="1"/>
-    <col min="32" max="32" width="14.28515625" style="10" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="51.5703125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="60.7109375" style="13" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" style="13" customWidth="1"/>
+    <col min="6" max="6" width="34.42578125" style="13" customWidth="1"/>
+    <col min="7" max="7" width="30.42578125" style="13" customWidth="1"/>
+    <col min="8" max="9" width="19.28515625" style="13" customWidth="1"/>
+    <col min="10" max="23" width="4.7109375" style="13" customWidth="1"/>
+    <col min="24" max="24" width="19.28515625" style="13" customWidth="1"/>
+    <col min="25" max="27" width="4.7109375" style="13" customWidth="1"/>
+    <col min="28" max="28" width="19.28515625" style="13" customWidth="1"/>
+    <col min="29" max="29" width="16.42578125" style="13" customWidth="1"/>
+    <col min="30" max="30" width="13.42578125" style="8" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="14.28515625" style="13" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="14.28515625" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="77" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="69"/>
-      <c r="S2" s="69"/>
-      <c r="T2" s="69"/>
-      <c r="U2" s="69"/>
-      <c r="V2" s="69"/>
-      <c r="W2" s="69"/>
-      <c r="X2" s="69"/>
-      <c r="Y2" s="69"/>
-      <c r="Z2" s="69"/>
-      <c r="AA2" s="69"/>
-      <c r="AB2" s="69"/>
-      <c r="AC2" s="69"/>
-      <c r="AD2" s="69"/>
-      <c r="AE2" s="69"/>
-      <c r="AF2" s="69"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
+      <c r="L2" s="77"/>
+      <c r="M2" s="77"/>
+      <c r="N2" s="77"/>
+      <c r="O2" s="77"/>
+      <c r="P2" s="77"/>
+      <c r="Q2" s="77"/>
+      <c r="R2" s="77"/>
+      <c r="S2" s="77"/>
+      <c r="T2" s="77"/>
+      <c r="U2" s="77"/>
+      <c r="V2" s="77"/>
+      <c r="W2" s="77"/>
+      <c r="X2" s="77"/>
+      <c r="Y2" s="77"/>
+      <c r="Z2" s="77"/>
+      <c r="AA2" s="77"/>
+      <c r="AB2" s="77"/>
+      <c r="AC2" s="77"/>
+      <c r="AD2" s="77"/>
+      <c r="AE2" s="77"/>
+      <c r="AF2" s="77"/>
     </row>
     <row r="3" spans="1:34" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="6"/>
-      <c r="Z3" s="6"/>
-      <c r="AA3" s="6"/>
-      <c r="AB3" s="6"/>
-      <c r="AC3" s="6"/>
-      <c r="AD3" s="6"/>
-      <c r="AE3" s="6"/>
-      <c r="AF3" s="11"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+      <c r="U3" s="9"/>
+      <c r="V3" s="9"/>
+      <c r="W3" s="9"/>
+      <c r="X3" s="9"/>
+      <c r="Y3" s="9"/>
+      <c r="Z3" s="9"/>
+      <c r="AA3" s="9"/>
+      <c r="AB3" s="9"/>
+      <c r="AC3" s="9"/>
+      <c r="AD3" s="9"/>
+      <c r="AE3" s="9"/>
+      <c r="AF3" s="14"/>
     </row>
     <row r="4" spans="1:34" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="12"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="70" t="s">
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="78" t="s">
         <v>99</v>
       </c>
-      <c r="K4" s="71"/>
-      <c r="L4" s="71"/>
-      <c r="M4" s="71"/>
-      <c r="N4" s="71"/>
-      <c r="O4" s="71"/>
-      <c r="P4" s="72"/>
-      <c r="Q4" s="70" t="s">
+      <c r="K4" s="79"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
+      <c r="N4" s="79"/>
+      <c r="O4" s="79"/>
+      <c r="P4" s="80"/>
+      <c r="Q4" s="78" t="s">
         <v>142</v>
       </c>
-      <c r="R4" s="71"/>
-      <c r="S4" s="71"/>
-      <c r="T4" s="71"/>
-      <c r="U4" s="71"/>
-      <c r="V4" s="71"/>
-      <c r="W4" s="72"/>
-      <c r="X4" s="12"/>
-      <c r="Y4" s="70" t="s">
+      <c r="R4" s="79"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="79"/>
+      <c r="U4" s="79"/>
+      <c r="V4" s="79"/>
+      <c r="W4" s="80"/>
+      <c r="X4" s="15"/>
+      <c r="Y4" s="78" t="s">
         <v>63</v>
       </c>
-      <c r="Z4" s="71"/>
-      <c r="AA4" s="72"/>
-      <c r="AB4" s="12"/>
-      <c r="AC4" s="12"/>
-      <c r="AD4" s="12"/>
-      <c r="AE4" s="12"/>
-      <c r="AF4" s="73" t="s">
+      <c r="Z4" s="79"/>
+      <c r="AA4" s="80"/>
+      <c r="AB4" s="15"/>
+      <c r="AC4" s="15"/>
+      <c r="AD4" s="15"/>
+      <c r="AE4" s="15"/>
+      <c r="AF4" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="AG4" s="74"/>
-      <c r="AH4" s="75"/>
-    </row>
-    <row r="5" spans="1:34" s="13" customFormat="1" ht="86.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="AG4" s="82"/>
+      <c r="AH4" s="83"/>
+    </row>
+    <row r="5" spans="1:34" s="16" customFormat="1" ht="86.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="I5" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="J5" s="15" t="s">
+      <c r="J5" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="K5" s="15" t="s">
+      <c r="K5" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="L5" s="15" t="s">
+      <c r="L5" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="M5" s="15" t="s">
+      <c r="M5" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="N5" s="15" t="s">
+      <c r="N5" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="O5" s="15" t="s">
+      <c r="O5" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="P5" s="15" t="s">
+      <c r="P5" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="Q5" s="15" t="s">
+      <c r="Q5" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="R5" s="15" t="s">
+      <c r="R5" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="S5" s="15" t="s">
+      <c r="S5" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="T5" s="15" t="s">
+      <c r="T5" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="U5" s="15" t="s">
+      <c r="U5" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="V5" s="15" t="s">
+      <c r="V5" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="W5" s="15" t="s">
+      <c r="W5" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="X5" s="14" t="s">
+      <c r="X5" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="Y5" s="15" t="s">
+      <c r="Y5" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="Z5" s="15" t="s">
+      <c r="Z5" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="AA5" s="15" t="s">
+      <c r="AA5" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="AB5" s="14" t="s">
+      <c r="AB5" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="AC5" s="14" t="s">
+      <c r="AC5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="AD5" s="14" t="s">
+      <c r="AD5" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="AE5" s="14" t="s">
+      <c r="AE5" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="AF5" s="14" t="s">
+      <c r="AF5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="AG5" s="16" t="s">
+      <c r="AG5" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="AH5" s="16" t="s">
+      <c r="AH5" s="19" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:34" s="5" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:34" s="8" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A6" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="I6" s="18" t="s">
+      <c r="I6" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="J6" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="Q6" s="19" t="s">
+      <c r="Q6" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="X6" s="19" t="s">
+      <c r="X6" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="AA6" s="19" t="s">
+      <c r="AA6" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="AB6" s="19" t="s">
+      <c r="AB6" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="AC6" s="19" t="s">
+      <c r="AC6" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="AF6" s="20" t="s">
+      <c r="AF6" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="AH6" s="21" t="s">
+      <c r="AH6" s="24" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:34" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="22" t="s">
+    <row r="7" spans="1:34" s="4" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="I7" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="J7" s="24" t="s">
+      <c r="J7" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="Q7" s="24" t="s">
+      <c r="Q7" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="X7" s="24" t="s">
+      <c r="X7" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="AA7" s="24" t="s">
+      <c r="AA7" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AB7" s="24" t="s">
+      <c r="AB7" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="AC7" s="24" t="s">
+      <c r="AC7" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AF7" s="25" t="s">
+      <c r="AF7" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AH7" s="26" t="s">
+      <c r="AH7" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:34" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A8" s="22" t="s">
+    <row r="8" spans="1:34" s="4" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="D8" s="23" t="s">
+      <c r="D8" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F8" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="G8" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="I8" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="J8" s="24" t="s">
+      <c r="J8" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="Q8" s="24" t="s">
+      <c r="Q8" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="X8" s="24" t="s">
+      <c r="X8" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="AA8" s="24" t="s">
+      <c r="AA8" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AB8" s="24" t="s">
+      <c r="AB8" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="AC8" s="24" t="s">
+      <c r="AC8" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AF8" s="25" t="s">
+      <c r="AF8" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AH8" s="26" t="s">
+      <c r="AH8" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="9" spans="1:34" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="22" t="s">
+    <row r="9" spans="1:34" s="4" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A9" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="J9" s="24" t="s">
+      <c r="J9" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="Q9" s="24" t="s">
+      <c r="Q9" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="X9" s="24" t="s">
+      <c r="X9" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="AA9" s="24" t="s">
+      <c r="AA9" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AB9" s="24" t="s">
+      <c r="AB9" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="AC9" s="24" t="s">
+      <c r="AC9" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AF9" s="25" t="s">
+      <c r="AF9" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AH9" s="26" t="s">
+      <c r="AH9" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:34" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
+    <row r="10" spans="1:34" s="4" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A10" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I10" s="23" t="s">
+      <c r="I10" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="J10" s="24" t="s">
+      <c r="J10" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="Q10" s="24" t="s">
+      <c r="Q10" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="X10" s="24" t="s">
+      <c r="X10" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="AA10" s="24" t="s">
+      <c r="AA10" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AB10" s="24" t="s">
+      <c r="AB10" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="AC10" s="24" t="s">
+      <c r="AC10" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AF10" s="25" t="s">
+      <c r="AF10" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AH10" s="26" t="s">
+      <c r="AH10" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:34" s="1" customFormat="1" ht="102" x14ac:dyDescent="0.2">
-      <c r="A11" s="22" t="s">
+    <row r="11" spans="1:34" s="4" customFormat="1" ht="102" x14ac:dyDescent="0.2">
+      <c r="A11" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="F11" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="G11" s="24" t="s">
+      <c r="G11" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H11" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I11" s="23" t="s">
+      <c r="I11" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="J11" s="24" t="s">
+      <c r="J11" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="Q11" s="24" t="s">
+      <c r="Q11" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="X11" s="24" t="s">
+      <c r="X11" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="AA11" s="24" t="s">
+      <c r="AA11" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AB11" s="24" t="s">
+      <c r="AB11" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="AC11" s="24" t="s">
+      <c r="AC11" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AF11" s="25" t="s">
+      <c r="AF11" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AH11" s="26" t="s">
+      <c r="AH11" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="12" spans="1:34" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="22" t="s">
+    <row r="12" spans="1:34" s="4" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="23" t="s">
+      <c r="F12" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="G12" s="24" t="s">
+      <c r="G12" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I12" s="23" t="s">
+      <c r="I12" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="J12" s="24" t="s">
+      <c r="J12" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="Q12" s="24" t="s">
+      <c r="Q12" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="X12" s="24" t="s">
+      <c r="X12" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="AA12" s="24" t="s">
+      <c r="AA12" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AB12" s="24" t="s">
+      <c r="AB12" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="AC12" s="24" t="s">
+      <c r="AC12" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AF12" s="25" t="s">
+      <c r="AF12" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AH12" s="26" t="s">
+      <c r="AH12" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="13" spans="1:34" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A13" s="22" t="s">
+    <row r="13" spans="1:34" s="4" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="G13" s="24" t="s">
+      <c r="G13" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I13" s="23" t="s">
+      <c r="I13" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="J13" s="24" t="s">
+      <c r="J13" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="Q13" s="24" t="s">
+      <c r="Q13" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="X13" s="24" t="s">
+      <c r="X13" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="AA13" s="24" t="s">
+      <c r="AA13" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AB13" s="24" t="s">
+      <c r="AB13" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="AC13" s="24" t="s">
+      <c r="AC13" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AF13" s="25" t="s">
+      <c r="AF13" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AH13" s="26" t="s">
+      <c r="AH13" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:34" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A14" s="22" t="s">
+    <row r="14" spans="1:34" s="4" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A14" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="23" t="s">
+      <c r="F14" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="24" t="s">
+      <c r="G14" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H14" s="24" t="s">
+      <c r="H14" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I14" s="23" t="s">
+      <c r="I14" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="J14" s="24" t="s">
+      <c r="J14" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="Q14" s="24" t="s">
+      <c r="Q14" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="X14" s="24" t="s">
+      <c r="X14" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="AA14" s="24" t="s">
+      <c r="AA14" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AB14" s="24" t="s">
+      <c r="AB14" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="AC14" s="24" t="s">
+      <c r="AC14" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AF14" s="25" t="s">
+      <c r="AF14" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AH14" s="26" t="s">
+      <c r="AH14" s="29" t="s">
         <v>87</v>
       </c>
     </row>
@@ -3072,603 +3075,584 @@
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" style="27" customWidth="1"/>
-    <col min="4" max="4" width="79.42578125" style="23" customWidth="1"/>
-    <col min="5" max="5" width="34.140625" style="28" customWidth="1"/>
-    <col min="6" max="6" width="35.7109375" style="28" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" style="30" customWidth="1"/>
+    <col min="4" max="4" width="79.42578125" style="26" customWidth="1"/>
+    <col min="5" max="5" width="34.140625" style="31" customWidth="1"/>
+    <col min="6" max="6" width="35.7109375" style="31" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
     </row>
     <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="B3" s="6"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-    </row>
-    <row r="4" spans="1:10" s="5" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="B4" s="33" t="s">
+      <c r="B3" s="9"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+    </row>
+    <row r="4" spans="1:10" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="B4" s="36" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="93" t="s">
+      <c r="C4" s="118" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="94"/>
-      <c r="E4" s="34" t="s">
+      <c r="D4" s="119"/>
+      <c r="E4" s="37" t="s">
         <v>157</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="F4" s="37" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="92" t="s">
+    <row r="5" spans="1:10" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="117" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="84" t="s">
+      <c r="C5" s="113" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="85"/>
-      <c r="E5" s="36" t="s">
+      <c r="D5" s="114"/>
+      <c r="E5" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="F5" s="37" t="s">
+      <c r="F5" s="40" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="92"/>
-      <c r="B6" s="35" t="s">
+    <row r="6" spans="1:10" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="117"/>
+      <c r="B6" s="38" t="s">
         <v>158</v>
       </c>
-      <c r="C6" s="84" t="s">
+      <c r="C6" s="113" t="s">
         <v>83</v>
       </c>
-      <c r="D6" s="85"/>
-      <c r="E6" s="38" t="s">
+      <c r="D6" s="114"/>
+      <c r="E6" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="F6" s="39" t="s">
+      <c r="F6" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="92"/>
-      <c r="B7" s="35" t="s">
+    <row r="7" spans="1:10" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="117"/>
+      <c r="B7" s="38" t="s">
         <v>136</v>
       </c>
-      <c r="C7" s="84" t="s">
+      <c r="C7" s="113" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="85"/>
-      <c r="E7" s="38" t="s">
+      <c r="D7" s="114"/>
+      <c r="E7" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="F7" s="39" t="s">
+      <c r="F7" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="92"/>
-      <c r="B8" s="40" t="s">
+    <row r="8" spans="1:10" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="117"/>
+      <c r="B8" s="43" t="s">
         <v>93</v>
       </c>
-      <c r="C8" s="86" t="s">
+      <c r="C8" s="100" t="s">
         <v>146</v>
       </c>
-      <c r="D8" s="87"/>
-      <c r="E8" s="38" t="s">
+      <c r="D8" s="101"/>
+      <c r="E8" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="F8" s="39" t="s">
+      <c r="F8" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="53.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="92"/>
-      <c r="B9" s="40" t="s">
+    <row r="9" spans="1:10" s="4" customFormat="1" ht="53.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="117"/>
+      <c r="B9" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="86" t="s">
+      <c r="C9" s="100" t="s">
         <v>151</v>
       </c>
-      <c r="D9" s="87"/>
-      <c r="E9" s="41" t="s">
+      <c r="D9" s="101"/>
+      <c r="E9" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="F9" s="39" t="s">
+      <c r="F9" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="10" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="92"/>
-      <c r="B10" s="35" t="s">
+    <row r="10" spans="1:10" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="117"/>
+      <c r="B10" s="38" t="s">
         <v>116</v>
       </c>
-      <c r="C10" s="88" t="s">
+      <c r="C10" s="104" t="s">
         <v>90</v>
       </c>
-      <c r="D10" s="91"/>
-      <c r="E10" s="38" t="s">
+      <c r="D10" s="105"/>
+      <c r="E10" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="F10" s="39" t="s">
+      <c r="F10" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="92"/>
-      <c r="B11" s="35" t="s">
+    <row r="11" spans="1:10" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="117"/>
+      <c r="B11" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="C11" s="88" t="s">
+      <c r="C11" s="104" t="s">
         <v>144</v>
       </c>
-      <c r="D11" s="89"/>
-      <c r="E11" s="41" t="s">
+      <c r="D11" s="115"/>
+      <c r="E11" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="41" t="s">
+      <c r="F11" s="44" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:10" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="92"/>
-      <c r="B12" s="35" t="s">
+    <row r="12" spans="1:10" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="117"/>
+      <c r="B12" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="C12" s="88" t="s">
+      <c r="C12" s="104" t="s">
         <v>75</v>
       </c>
-      <c r="D12" s="91"/>
-      <c r="E12" s="38" t="s">
+      <c r="D12" s="105"/>
+      <c r="E12" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="F12" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="92"/>
-      <c r="B13" s="40" t="s">
+    <row r="13" spans="1:10" s="4" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="117"/>
+      <c r="B13" s="43" t="s">
         <v>133</v>
       </c>
-      <c r="C13" s="88" t="s">
+      <c r="C13" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="91"/>
-      <c r="E13" s="38" t="s">
+      <c r="D13" s="105"/>
+      <c r="E13" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="F13" s="39" t="s">
+      <c r="F13" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="14" spans="1:10" s="1" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="92"/>
-      <c r="B14" s="79" t="s">
+    <row r="14" spans="1:10" s="4" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="117"/>
+      <c r="B14" s="108" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="82" t="s">
+      <c r="C14" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="83"/>
-      <c r="E14" s="105" t="s">
+      <c r="D14" s="112"/>
+      <c r="E14" s="87" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="108" t="s">
+      <c r="F14" s="90" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="92"/>
-      <c r="B15" s="80"/>
-      <c r="C15" s="42" t="s">
+    <row r="15" spans="1:10" s="4" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="117"/>
+      <c r="B15" s="109"/>
+      <c r="C15" s="45" t="s">
         <v>138</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="26" t="s">
         <v>129</v>
       </c>
-      <c r="E15" s="106"/>
-      <c r="F15" s="109"/>
-    </row>
-    <row r="16" spans="1:10" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="92"/>
-      <c r="B16" s="80"/>
-      <c r="C16" s="42" t="s">
+      <c r="E15" s="88"/>
+      <c r="F15" s="91"/>
+    </row>
+    <row r="16" spans="1:10" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="117"/>
+      <c r="B16" s="109"/>
+      <c r="C16" s="45" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="106"/>
-      <c r="F16" s="109"/>
-    </row>
-    <row r="17" spans="1:6" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="92"/>
-      <c r="B17" s="80"/>
-      <c r="C17" s="42" t="s">
+      <c r="E16" s="88"/>
+      <c r="F16" s="91"/>
+    </row>
+    <row r="17" spans="1:6" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="117"/>
+      <c r="B17" s="109"/>
+      <c r="C17" s="45" t="s">
         <v>110</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="E17" s="106"/>
-      <c r="F17" s="109"/>
-    </row>
-    <row r="18" spans="1:6" s="1" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="92"/>
-      <c r="B18" s="80"/>
-      <c r="C18" s="42" t="s">
+      <c r="E17" s="88"/>
+      <c r="F17" s="91"/>
+    </row>
+    <row r="18" spans="1:6" s="4" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="117"/>
+      <c r="B18" s="109"/>
+      <c r="C18" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="E18" s="106"/>
-      <c r="F18" s="109"/>
-    </row>
-    <row r="19" spans="1:6" s="1" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="92"/>
-      <c r="B19" s="80"/>
-      <c r="C19" s="42" t="s">
+      <c r="E18" s="88"/>
+      <c r="F18" s="91"/>
+    </row>
+    <row r="19" spans="1:6" s="4" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="117"/>
+      <c r="B19" s="109"/>
+      <c r="C19" s="45" t="s">
         <v>168</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="E19" s="106"/>
-      <c r="F19" s="109"/>
-    </row>
-    <row r="20" spans="1:6" s="1" customFormat="1" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="92"/>
-      <c r="B20" s="80"/>
-      <c r="C20" s="42" t="s">
+      <c r="E19" s="88"/>
+      <c r="F19" s="91"/>
+    </row>
+    <row r="20" spans="1:6" s="4" customFormat="1" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="117"/>
+      <c r="B20" s="109"/>
+      <c r="C20" s="45" t="s">
         <v>44</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="D20" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="E20" s="106"/>
-      <c r="F20" s="109"/>
-    </row>
-    <row r="21" spans="1:6" s="1" customFormat="1" ht="57.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="92"/>
-      <c r="B21" s="81"/>
-      <c r="C21" s="42" t="s">
+      <c r="E20" s="88"/>
+      <c r="F20" s="91"/>
+    </row>
+    <row r="21" spans="1:6" s="4" customFormat="1" ht="57.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="117"/>
+      <c r="B21" s="110"/>
+      <c r="C21" s="45" t="s">
         <v>117</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="E21" s="107"/>
-      <c r="F21" s="110"/>
-    </row>
-    <row r="22" spans="1:6" s="1" customFormat="1" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="92"/>
-      <c r="B22" s="90" t="s">
+      <c r="E21" s="89"/>
+      <c r="F21" s="92"/>
+    </row>
+    <row r="22" spans="1:6" s="4" customFormat="1" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="117"/>
+      <c r="B22" s="116" t="s">
         <v>142</v>
       </c>
-      <c r="C22" s="98" t="s">
+      <c r="C22" s="102" t="s">
         <v>71</v>
       </c>
-      <c r="D22" s="99"/>
-      <c r="E22" s="105" t="s">
+      <c r="D22" s="103"/>
+      <c r="E22" s="87" t="s">
         <v>49</v>
       </c>
-      <c r="F22" s="108" t="s">
+      <c r="F22" s="90" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="23" spans="1:6" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="92"/>
-      <c r="B23" s="80"/>
-      <c r="C23" s="43" t="s">
+    <row r="23" spans="1:6" s="4" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="117"/>
+      <c r="B23" s="109"/>
+      <c r="C23" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="D23" s="23" t="s">
+      <c r="D23" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="E23" s="106"/>
-      <c r="F23" s="109"/>
-    </row>
-    <row r="24" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="92"/>
-      <c r="B24" s="80"/>
-      <c r="C24" s="43" t="s">
+      <c r="E23" s="88"/>
+      <c r="F23" s="91"/>
+    </row>
+    <row r="24" spans="1:6" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="117"/>
+      <c r="B24" s="109"/>
+      <c r="C24" s="46" t="s">
         <v>150</v>
       </c>
-      <c r="D24" s="23" t="s">
+      <c r="D24" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="E24" s="106"/>
-      <c r="F24" s="109"/>
-    </row>
-    <row r="25" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="92"/>
-      <c r="B25" s="80"/>
-      <c r="C25" s="43" t="s">
+      <c r="E24" s="88"/>
+      <c r="F24" s="91"/>
+    </row>
+    <row r="25" spans="1:6" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="117"/>
+      <c r="B25" s="109"/>
+      <c r="C25" s="46" t="s">
         <v>115</v>
       </c>
-      <c r="D25" s="23" t="s">
+      <c r="D25" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="E25" s="106"/>
-      <c r="F25" s="109"/>
-    </row>
-    <row r="26" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="92"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="43" t="s">
+      <c r="E25" s="88"/>
+      <c r="F25" s="91"/>
+    </row>
+    <row r="26" spans="1:6" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="117"/>
+      <c r="B26" s="109"/>
+      <c r="C26" s="46" t="s">
         <v>154</v>
       </c>
-      <c r="D26" s="23" t="s">
+      <c r="D26" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="E26" s="106"/>
-      <c r="F26" s="109"/>
-    </row>
-    <row r="27" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="92"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="43" t="s">
+      <c r="E26" s="88"/>
+      <c r="F26" s="91"/>
+    </row>
+    <row r="27" spans="1:6" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="117"/>
+      <c r="B27" s="109"/>
+      <c r="C27" s="46" t="s">
         <v>169</v>
       </c>
-      <c r="D27" s="44" t="s">
+      <c r="D27" s="47" t="s">
         <v>118</v>
       </c>
-      <c r="E27" s="106"/>
-      <c r="F27" s="109"/>
-    </row>
-    <row r="28" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="92"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="43" t="s">
+      <c r="E27" s="88"/>
+      <c r="F27" s="91"/>
+    </row>
+    <row r="28" spans="1:6" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="117"/>
+      <c r="B28" s="109"/>
+      <c r="C28" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="D28" s="44" t="s">
+      <c r="D28" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="E28" s="106"/>
-      <c r="F28" s="109"/>
-    </row>
-    <row r="29" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="92"/>
-      <c r="B29" s="81"/>
-      <c r="C29" s="45" t="s">
+      <c r="E28" s="88"/>
+      <c r="F28" s="91"/>
+    </row>
+    <row r="29" spans="1:6" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="117"/>
+      <c r="B29" s="110"/>
+      <c r="C29" s="48" t="s">
         <v>123</v>
       </c>
-      <c r="D29" s="46" t="s">
+      <c r="D29" s="49" t="s">
         <v>108</v>
       </c>
-      <c r="E29" s="107"/>
-      <c r="F29" s="110"/>
-    </row>
-    <row r="30" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="92"/>
-      <c r="B30" s="47" t="s">
+      <c r="E29" s="89"/>
+      <c r="F29" s="92"/>
+    </row>
+    <row r="30" spans="1:6" s="4" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="117"/>
+      <c r="B30" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="C30" s="100" t="s">
+      <c r="C30" s="106" t="s">
         <v>153</v>
       </c>
-      <c r="D30" s="101"/>
-      <c r="E30" s="41" t="s">
+      <c r="D30" s="107"/>
+      <c r="E30" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="F30" s="39" t="s">
+      <c r="F30" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="31" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="92"/>
-      <c r="B31" s="76" t="s">
+    <row r="31" spans="1:6" s="4" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="117"/>
+      <c r="B31" s="95" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="88" t="s">
+      <c r="C31" s="104" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="91"/>
-      <c r="E31" s="105" t="s">
+      <c r="D31" s="105"/>
+      <c r="E31" s="87" t="s">
         <v>49</v>
       </c>
-      <c r="F31" s="108" t="s">
+      <c r="F31" s="90" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="32" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="92"/>
-      <c r="B32" s="77"/>
-      <c r="C32" s="48" t="s">
+    <row r="32" spans="1:6" s="4" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="117"/>
+      <c r="B32" s="96"/>
+      <c r="C32" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="D32" s="49" t="s">
+      <c r="D32" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="E32" s="106"/>
-      <c r="F32" s="109"/>
-    </row>
-    <row r="33" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="92"/>
-      <c r="B33" s="77"/>
-      <c r="C33" s="48" t="s">
+      <c r="E32" s="88"/>
+      <c r="F32" s="91"/>
+    </row>
+    <row r="33" spans="1:6" s="4" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="117"/>
+      <c r="B33" s="96"/>
+      <c r="C33" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="D33" s="50" t="s">
+      <c r="D33" s="53" t="s">
         <v>149</v>
       </c>
-      <c r="E33" s="106"/>
-      <c r="F33" s="109"/>
-    </row>
-    <row r="34" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="92"/>
-      <c r="B34" s="78"/>
-      <c r="C34" s="48" t="s">
+      <c r="E33" s="88"/>
+      <c r="F33" s="91"/>
+    </row>
+    <row r="34" spans="1:6" s="4" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="117"/>
+      <c r="B34" s="97"/>
+      <c r="C34" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D34" s="50" t="s">
+      <c r="D34" s="53" t="s">
         <v>65</v>
       </c>
-      <c r="E34" s="107"/>
-      <c r="F34" s="110"/>
-    </row>
-    <row r="35" spans="1:6" s="1" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="95" t="s">
+      <c r="E34" s="89"/>
+      <c r="F34" s="92"/>
+    </row>
+    <row r="35" spans="1:6" s="4" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="94" t="s">
         <v>77</v>
       </c>
-      <c r="B35" s="35" t="s">
+      <c r="B35" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C35" s="88" t="s">
+      <c r="C35" s="104" t="s">
         <v>85</v>
       </c>
-      <c r="D35" s="91"/>
-      <c r="E35" s="38" t="s">
+      <c r="D35" s="105"/>
+      <c r="E35" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="F35" s="39" t="s">
+      <c r="F35" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="36" spans="1:6" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="95"/>
-      <c r="B36" s="35" t="s">
+    <row r="36" spans="1:6" s="4" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="94"/>
+      <c r="B36" s="38" t="s">
         <v>161</v>
       </c>
-      <c r="C36" s="88" t="s">
+      <c r="C36" s="104" t="s">
         <v>37</v>
       </c>
-      <c r="D36" s="91"/>
-      <c r="E36" s="38" t="s">
+      <c r="D36" s="105"/>
+      <c r="E36" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="F36" s="39" t="s">
+      <c r="F36" s="42" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="37" spans="1:6" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="95"/>
-      <c r="B37" s="76" t="s">
+    <row r="37" spans="1:6" s="4" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="94"/>
+      <c r="B37" s="95" t="s">
         <v>33</v>
       </c>
-      <c r="C37" s="96" t="s">
+      <c r="C37" s="98" t="s">
         <v>121</v>
       </c>
-      <c r="D37" s="97"/>
-      <c r="E37" s="102" t="s">
+      <c r="D37" s="99"/>
+      <c r="E37" s="84" t="s">
         <v>135</v>
       </c>
-      <c r="F37" s="108" t="s">
+      <c r="F37" s="90" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="38" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="95"/>
-      <c r="B38" s="77"/>
-      <c r="C38" s="43" t="s">
+    <row r="38" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="94"/>
+      <c r="B38" s="96"/>
+      <c r="C38" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="44" t="s">
+      <c r="D38" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="103"/>
-      <c r="F38" s="109"/>
-    </row>
-    <row r="39" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="95"/>
-      <c r="B39" s="77"/>
-      <c r="C39" s="43" t="s">
+      <c r="E38" s="85"/>
+      <c r="F38" s="91"/>
+    </row>
+    <row r="39" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="94"/>
+      <c r="B39" s="96"/>
+      <c r="C39" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="D39" s="23" t="s">
+      <c r="D39" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="E39" s="103"/>
-      <c r="F39" s="109"/>
-    </row>
-    <row r="40" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="95"/>
-      <c r="B40" s="77"/>
-      <c r="C40" s="43" t="s">
+      <c r="E39" s="85"/>
+      <c r="F39" s="91"/>
+    </row>
+    <row r="40" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="94"/>
+      <c r="B40" s="96"/>
+      <c r="C40" s="46" t="s">
         <v>139</v>
       </c>
-      <c r="D40" s="44" t="s">
+      <c r="D40" s="47" t="s">
         <v>97</v>
       </c>
-      <c r="E40" s="103"/>
-      <c r="F40" s="109"/>
-    </row>
-    <row r="41" spans="1:6" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A41" s="95"/>
-      <c r="B41" s="77"/>
-      <c r="C41" s="43" t="s">
+      <c r="E40" s="85"/>
+      <c r="F40" s="91"/>
+    </row>
+    <row r="41" spans="1:6" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A41" s="94"/>
+      <c r="B41" s="96"/>
+      <c r="C41" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="D41" s="23" t="s">
+      <c r="D41" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="E41" s="103"/>
-      <c r="F41" s="109"/>
-    </row>
-    <row r="42" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="95"/>
-      <c r="B42" s="78"/>
-      <c r="C42" s="51" t="s">
+      <c r="E41" s="85"/>
+      <c r="F41" s="91"/>
+    </row>
+    <row r="42" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="94"/>
+      <c r="B42" s="97"/>
+      <c r="C42" s="54" t="s">
         <v>57</v>
       </c>
-      <c r="D42" s="46" t="s">
+      <c r="D42" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="E42" s="104"/>
-      <c r="F42" s="111"/>
+      <c r="E42" s="86"/>
+      <c r="F42" s="93"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="E37:E42"/>
-    <mergeCell ref="E31:E34"/>
-    <mergeCell ref="E22:E29"/>
-    <mergeCell ref="E14:E21"/>
-    <mergeCell ref="F14:F21"/>
-    <mergeCell ref="F22:F29"/>
-    <mergeCell ref="F37:F42"/>
-    <mergeCell ref="F31:F34"/>
-    <mergeCell ref="A35:A42"/>
-    <mergeCell ref="B37:B42"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C12:D12"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B31:B34"/>
     <mergeCell ref="B14:B21"/>
@@ -3682,6 +3666,25 @@
     <mergeCell ref="A5:A34"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A35:A42"/>
+    <mergeCell ref="B37:B42"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E37:E42"/>
+    <mergeCell ref="E31:E34"/>
+    <mergeCell ref="E22:E29"/>
+    <mergeCell ref="E14:E21"/>
+    <mergeCell ref="F14:F21"/>
+    <mergeCell ref="F22:F29"/>
+    <mergeCell ref="F37:F42"/>
+    <mergeCell ref="F31:F34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -3693,156 +3696,164 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="10" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="54.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="54.42578125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="112" t="s">
+      <c r="A3" s="120" t="s">
         <v>66</v>
       </c>
-      <c r="B3" s="112"/>
-      <c r="C3" s="112"/>
-      <c r="D3" s="113"/>
+      <c r="B3" s="120"/>
+      <c r="C3" s="120"/>
+      <c r="D3" s="121"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="114"/>
-      <c r="B4" s="114"/>
-      <c r="C4" s="114"/>
-      <c r="D4" s="115"/>
+      <c r="A4" s="122"/>
+      <c r="B4" s="122"/>
+      <c r="C4" s="122"/>
+      <c r="D4" s="123"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="116"/>
-      <c r="B5" s="116"/>
-      <c r="C5" s="116"/>
-      <c r="D5" s="117"/>
+      <c r="A5" s="124"/>
+      <c r="B5" s="124"/>
+      <c r="C5" s="124"/>
+      <c r="D5" s="125"/>
     </row>
     <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="52" t="s">
+      <c r="B6" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="52" t="s">
+      <c r="D6" s="55" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="53"/>
-      <c r="B7" s="54"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="53"/>
+      <c r="A7" s="56"/>
+      <c r="B7" s="57"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="56"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="53"/>
-      <c r="B8" s="54"/>
-      <c r="C8" s="55"/>
-      <c r="D8" s="53"/>
+      <c r="A8" s="56"/>
+      <c r="B8" s="57"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="56"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="53"/>
-      <c r="B9" s="54"/>
-      <c r="C9" s="55"/>
-      <c r="D9" s="53"/>
+      <c r="A9" s="56"/>
+      <c r="B9" s="57"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="56"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="53"/>
-      <c r="B10" s="54"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="53"/>
+      <c r="A10" s="56"/>
+      <c r="B10" s="57"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="56"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="112" t="s">
+      <c r="A15" s="120" t="s">
         <v>126</v>
       </c>
-      <c r="B15" s="112"/>
-      <c r="C15" s="112"/>
-      <c r="D15" s="113"/>
+      <c r="B15" s="120"/>
+      <c r="C15" s="120"/>
+      <c r="D15" s="121"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="114"/>
-      <c r="B16" s="114"/>
-      <c r="C16" s="114"/>
-      <c r="D16" s="115"/>
+      <c r="A16" s="122"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="123"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="116"/>
-      <c r="B17" s="116"/>
-      <c r="C17" s="116"/>
-      <c r="D17" s="117"/>
+      <c r="A17" s="124"/>
+      <c r="B17" s="124"/>
+      <c r="C17" s="124"/>
+      <c r="D17" s="125"/>
     </row>
     <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="52" t="s">
+      <c r="A18" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="52" t="s">
+      <c r="B18" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="C18" s="52" t="s">
+      <c r="C18" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="52" t="s">
+      <c r="D18" s="55" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="53" t="s">
+      <c r="A19" s="56" t="s">
         <v>132</v>
       </c>
-      <c r="B19" s="54" t="s">
+      <c r="B19" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="55">
+      <c r="C19" s="58">
         <v>43343</v>
       </c>
-      <c r="D19" s="53" t="s">
+      <c r="D19" s="56" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A20" s="53" t="s">
+      <c r="A20" s="56" t="s">
         <v>132</v>
       </c>
-      <c r="B20" s="54" t="s">
+      <c r="B20" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="C20" s="55">
+      <c r="C20" s="58">
         <v>43396</v>
       </c>
-      <c r="D20" s="53" t="s">
+      <c r="D20" s="56" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="127.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="53" t="s">
+      <c r="A21" s="56" t="s">
         <v>132</v>
       </c>
-      <c r="B21" s="54" t="s">
+      <c r="B21" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="C21" s="55">
+      <c r="C21" s="58">
         <v>43413</v>
       </c>
-      <c r="D21" s="53" t="s">
+      <c r="D21" s="56" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="53"/>
-      <c r="B22" s="54"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="53"/>
+    <row r="22" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A22" s="56" t="s">
+        <v>173</v>
+      </c>
+      <c r="B22" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="C22" s="58">
+        <v>43557</v>
+      </c>
+      <c r="D22" s="56" t="s">
+        <v>175</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
docs - Test report and traceability
Signed-off-by: Prasad Jondhale <prasad.jondhale@ti.com>
</commit_message>
<xml_diff>
--- a/docs/test_report/ethfw_testreport.xlsx
+++ b/docs/test_report/ethfw_testreport.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-12" yWindow="0" windowWidth="12300" windowHeight="2616" tabRatio="599"/>
+    <workbookView xWindow="12840" yWindow="0" windowWidth="13725" windowHeight="8355" tabRatio="599"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Revision History" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Details'!$A$5:$AF$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Details'!$A$5:$AD$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Revision History'!#REF!</definedName>
     <definedName name="Test_Category">Help!#REF!</definedName>
   </definedNames>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="180">
   <si>
     <t>Test is not required for this release (e.g., test case not supported for targeted platform)</t>
   </si>
@@ -42,9 +42,6 @@
     <t>Test Case covers usability/api/look and feel aspects of the module including out-of box (OOB) experience</t>
   </si>
   <si>
-    <t>Switching on all external ports on VLAB</t>
-  </si>
-  <si>
     <t>This fields identifies whether the test is part of regression to verify software changes, or part of full software test cycle.</t>
   </si>
   <si>
@@ -102,6 +99,12 @@
     <t>Category</t>
   </si>
   <si>
+    <t>EthFW Protocol Test - NDK integration</t>
+  </si>
+  <si>
+    <t>ETHFW-385</t>
+  </si>
+  <si>
     <t>Test cases derived by division of inputs and outputs ranges to ensure a representative test value can be selected for each class or range.</t>
   </si>
   <si>
@@ -141,9 +144,6 @@
     <t>ETHFW-37 : [EthFW][System]Driver Integration:UART: UART driver should be integrated and used for development time log prints</t>
   </si>
   <si>
-    <t>[EthFW]Switching on all external ports on VLAB</t>
-  </si>
-  <si>
     <t>Test Blocked because of other test case failure, an Open MR from previous Release, feature not implemented yet, feature not supported by hardware</t>
   </si>
   <si>
@@ -198,9 +198,6 @@
     <t>NRQ</t>
   </si>
   <si>
-    <t>ETHFW-181 : [EthFW]Switching on all external ports on VLAB</t>
-  </si>
-  <si>
     <t>X</t>
   </si>
   <si>
@@ -240,13 +237,10 @@
     <t>As part of test planning, various methods are used to derive test cases.  This field identifies the test derivation method was associated with this test case.  The possible derivation methods are defined below:</t>
   </si>
   <si>
-    <t>'J7-PRESI'</t>
+    <t>J7-EVM</t>
   </si>
   <si>
     <t>ETHFW-56 : [EthFW][OS]OS:cpsw_lld should be validated on  split mode variant of TI RTOS config</t>
-  </si>
-  <si>
-    <t>J7-PRESI</t>
   </si>
   <si>
     <t>Clean-up.  Removed some tabs that were erroneously left in by mistake.</t>
@@ -339,9 +333,6 @@
     <t>EthFW System Test - GPTIMER Driver Integration</t>
   </si>
   <si>
-    <t>All</t>
-  </si>
-  <si>
     <t>B</t>
   </si>
   <si>
@@ -358,6 +349,9 @@
     <t>Test cases established based on lessons learned and expert judgement to determine situations that may cause software failures or errors to appear</t>
   </si>
   <si>
+    <t>[EthFW][Protocol]Protocol: Switch resident protocol:NDK integration to enable TCP/UDP/ICMP/IP</t>
+  </si>
+  <si>
     <t>[EthFW][System]Driver Integration:UART: UART driver should be integrated and used for development time log prints</t>
   </si>
   <si>
@@ -454,21 +448,18 @@
     <t>Test cases derived to demonstrate intended functionality of the software derived from analysis of software requirements</t>
   </si>
   <si>
-    <t>ETHFW-182</t>
-  </si>
-  <si>
     <t>Test Derivation Method</t>
   </si>
   <si>
     <t>Successful execution of EThFw switching test with sysbios</t>
   </si>
   <si>
+    <t>'J7-EVM'</t>
+  </si>
+  <si>
     <t>Optional project-specific field that can be used to further classify specifc test area or module</t>
   </si>
   <si>
-    <t>ETHFW-178</t>
-  </si>
-  <si>
     <t>Functional Requirement ID(s) from the SPS that this test case covers (comma separated).  For automotive and functional safety, this may also include design ID and/or architecture IDs as well.</t>
   </si>
   <si>
@@ -476,6 +467,9 @@
   </si>
   <si>
     <t>Should successfully execute CPsw Switching App with Cpsw library linked with tirtos osal implementation</t>
+  </si>
+  <si>
+    <t>Should able to send/receive packets through TCP/UDP/ICMP/IP</t>
   </si>
   <si>
     <t>This Test case is identified to run for Regression / maintenance releases</t>
@@ -499,10 +493,16 @@
     <t>Use Case Analysis</t>
   </si>
   <si>
+    <t>ETHFW-386</t>
+  </si>
+  <si>
     <t>Test Case ensures that the component does not fail over time
 IEEE Defn: The ability of a system or component to perform its required functions under stated conditions for a specified period of time</t>
   </si>
   <si>
+    <t>ETHFW-64 : [EthFW][Protocol]Protocol: Switch resident protocol:NDK integration to enable TCP/UDP/ICMP/IP</t>
+  </si>
+  <si>
     <t>Test cases derived from analysis of potential error conditions</t>
   </si>
   <si>
@@ -527,9 +527,6 @@
     <t>ETHFW-156</t>
   </si>
   <si>
-    <t>4/3/2019</t>
-  </si>
-  <si>
     <t>[EthFW][OS]OS:cpsw_lld should be validated on split mode variant of TI RTOS config</t>
   </si>
   <si>
@@ -542,18 +539,21 @@
     <t>[EthFW][OS]OSAL:EMAC Osal:Baremetal implementation of EMAL osal interface should be integrated into the switch firmware</t>
   </si>
   <si>
+    <t>ETHFW-387</t>
+  </si>
+  <si>
     <t>Performance</t>
   </si>
   <si>
     <t>Customer Usage</t>
   </si>
   <si>
+    <t>7/18/2019</t>
+  </si>
+  <si>
     <t>Processor SDK Vision - EthFw</t>
   </si>
   <si>
-    <t>EthFw_J7_00.08.00_EA8</t>
-  </si>
-  <si>
     <t>Prasad Jondhale</t>
   </si>
   <si>
@@ -561,6 +561,18 @@
   </si>
   <si>
     <t>Downloaded from FoQus for 0.8 release and updated the summary tab and test details</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>Downloaded from FoQus for 0.9 release and updated the summary tab and test details</t>
+  </si>
+  <si>
+    <t>EthFw_J7_00.09.00_BRINGUP</t>
+  </si>
+  <si>
+    <t>TI-RTOS</t>
   </si>
 </sst>
 </file>
@@ -1536,12 +1548,24 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1682,18 +1706,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="48" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="49" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1703,74 +1715,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1832,7 +1776,7 @@
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="DBEEDD"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -2110,21 +2054,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="57" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C2" s="58"/>
       <c r="D2" s="58"/>
@@ -2134,12 +2078,12 @@
       <c r="H2" s="58"/>
       <c r="I2" s="59"/>
     </row>
-    <row r="3" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
     </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="63" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="64"/>
       <c r="C4" s="64"/>
@@ -2148,78 +2092,78 @@
       <c r="F4" s="64"/>
       <c r="G4" s="65"/>
     </row>
-    <row r="5" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="66" t="s">
-        <v>171</v>
-      </c>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
+        <v>172</v>
+      </c>
+      <c r="C5" s="67"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="67"/>
+      <c r="F5" s="67"/>
       <c r="G5" s="68"/>
     </row>
-    <row r="6" spans="1:9" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="B6" s="118" t="s">
-        <v>172</v>
-      </c>
-      <c r="C6" s="119"/>
-      <c r="D6" s="119"/>
-      <c r="E6" s="119"/>
-      <c r="F6" s="119"/>
-      <c r="G6" s="120"/>
-    </row>
-    <row r="7" spans="1:9" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="69" t="s">
+        <v>178</v>
+      </c>
+      <c r="C6" s="70"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="70"/>
+      <c r="F6" s="70"/>
+      <c r="G6" s="71"/>
+    </row>
+    <row r="7" spans="1:9" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="66" t="s">
-        <v>164</v>
-      </c>
-      <c r="C7" s="67"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
+        <v>171</v>
+      </c>
+      <c r="C7" s="72"/>
+      <c r="D7" s="72"/>
+      <c r="E7" s="72"/>
+      <c r="F7" s="72"/>
       <c r="G7" s="68"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
     </row>
-    <row r="8" spans="1:9" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="67"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
+        <v>141</v>
+      </c>
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
       <c r="G8" s="68"/>
     </row>
-    <row r="9" spans="1:9" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="67"/>
-      <c r="D9" s="67"/>
-      <c r="E9" s="67"/>
-      <c r="F9" s="67"/>
+        <v>179</v>
+      </c>
+      <c r="C9" s="72"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="72"/>
+      <c r="F9" s="72"/>
       <c r="G9" s="68"/>
     </row>
-    <row r="10" spans="1:9" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
     </row>
-    <row r="11" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="60" t="s">
         <v>3</v>
       </c>
@@ -2230,49 +2174,49 @@
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
     </row>
-    <row r="13" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B13" s="56" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C13" s="56"/>
     </row>
-    <row r="14" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" s="9">
         <v>9</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B15" s="9">
         <v>0</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16" s="9">
         <v>0</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>57</v>
       </c>
@@ -2280,18 +2224,18 @@
         <v>0</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" s="9">
         <v>0</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -2314,69 +2258,66 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AG14"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AE14"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="51.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="60.6640625" style="10" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" style="10" customWidth="1"/>
-    <col min="6" max="6" width="34.44140625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="30.44140625" style="10" customWidth="1"/>
-    <col min="8" max="9" width="19.33203125" style="10" customWidth="1"/>
-    <col min="10" max="23" width="4.6640625" style="10" customWidth="1"/>
-    <col min="24" max="24" width="19.33203125" style="10" customWidth="1"/>
-    <col min="25" max="27" width="4.6640625" style="10" customWidth="1"/>
-    <col min="28" max="28" width="19.33203125" style="10" customWidth="1"/>
-    <col min="29" max="29" width="16.44140625" style="10" customWidth="1"/>
-    <col min="30" max="30" width="13.44140625" style="5" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="14.33203125" style="10" hidden="1" customWidth="1"/>
-    <col min="32" max="32" width="14.33203125" style="10" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="51.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="60.7109375" style="10" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="34.42578125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" style="10" customWidth="1"/>
+    <col min="8" max="21" width="4.7109375" style="10" customWidth="1"/>
+    <col min="22" max="22" width="19.28515625" style="10" customWidth="1"/>
+    <col min="23" max="25" width="4.7109375" style="10" customWidth="1"/>
+    <col min="26" max="26" width="19.28515625" style="10" customWidth="1"/>
+    <col min="27" max="27" width="16.42578125" style="10" customWidth="1"/>
+    <col min="28" max="28" width="13.42578125" style="5" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="14.28515625" style="10" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="14.28515625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="69" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="69"/>
-      <c r="S2" s="69"/>
-      <c r="T2" s="69"/>
-      <c r="U2" s="69"/>
-      <c r="V2" s="69"/>
-      <c r="W2" s="69"/>
-      <c r="X2" s="69"/>
-      <c r="Y2" s="69"/>
-      <c r="Z2" s="69"/>
-      <c r="AA2" s="69"/>
-      <c r="AB2" s="69"/>
-      <c r="AC2" s="69"/>
-      <c r="AD2" s="69"/>
-      <c r="AE2" s="69"/>
-      <c r="AF2" s="69"/>
-    </row>
-    <row r="3" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="73" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
+      <c r="P2" s="73"/>
+      <c r="Q2" s="73"/>
+      <c r="R2" s="73"/>
+      <c r="S2" s="73"/>
+      <c r="T2" s="73"/>
+      <c r="U2" s="73"/>
+      <c r="V2" s="73"/>
+      <c r="W2" s="73"/>
+      <c r="X2" s="73"/>
+      <c r="Y2" s="73"/>
+      <c r="Z2" s="73"/>
+      <c r="AA2" s="73"/>
+      <c r="AB2" s="73"/>
+      <c r="AC2" s="73"/>
+      <c r="AD2" s="73"/>
+    </row>
+    <row r="3" spans="1:31" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -2406,11 +2347,9 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="6"/>
-      <c r="AE3" s="6"/>
-      <c r="AF3" s="11"/>
-    </row>
-    <row r="4" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AD3" s="11"/>
+    </row>
+    <row r="4" spans="1:31" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -2418,42 +2357,40 @@
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="70" t="s">
-        <v>100</v>
-      </c>
-      <c r="K4" s="71"/>
-      <c r="L4" s="71"/>
-      <c r="M4" s="71"/>
-      <c r="N4" s="71"/>
-      <c r="O4" s="71"/>
-      <c r="P4" s="72"/>
-      <c r="Q4" s="70" t="s">
-        <v>142</v>
-      </c>
-      <c r="R4" s="71"/>
-      <c r="S4" s="71"/>
-      <c r="T4" s="71"/>
-      <c r="U4" s="71"/>
-      <c r="V4" s="71"/>
-      <c r="W4" s="72"/>
-      <c r="X4" s="12"/>
-      <c r="Y4" s="70" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z4" s="71"/>
-      <c r="AA4" s="72"/>
+      <c r="H4" s="74" t="s">
+        <v>98</v>
+      </c>
+      <c r="I4" s="75"/>
+      <c r="J4" s="75"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="75"/>
+      <c r="M4" s="75"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="74" t="s">
+        <v>139</v>
+      </c>
+      <c r="P4" s="75"/>
+      <c r="Q4" s="75"/>
+      <c r="R4" s="75"/>
+      <c r="S4" s="75"/>
+      <c r="T4" s="75"/>
+      <c r="U4" s="76"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="74" t="s">
+        <v>62</v>
+      </c>
+      <c r="X4" s="75"/>
+      <c r="Y4" s="76"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="12"/>
       <c r="AB4" s="12"/>
       <c r="AC4" s="12"/>
-      <c r="AD4" s="12"/>
-      <c r="AE4" s="12"/>
-      <c r="AF4" s="73" t="s">
-        <v>33</v>
-      </c>
-      <c r="AG4" s="74"/>
-    </row>
-    <row r="5" spans="1:33" s="13" customFormat="1" ht="86.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AD4" s="77" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE4" s="78"/>
+    </row>
+    <row r="5" spans="1:31" s="13" customFormat="1" ht="86.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>51</v>
       </c>
@@ -2461,105 +2398,99 @@
         <v>158</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>54</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>120</v>
+        <v>118</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>42</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>111</v>
+        <v>169</v>
       </c>
       <c r="M5" s="15" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>169</v>
+        <v>115</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>44</v>
+        <v>150</v>
       </c>
       <c r="P5" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q5" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="R5" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="S5" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="T5" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="U5" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="V5" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="Q5" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="R5" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="S5" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="T5" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="U5" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="V5" s="15" t="s">
-        <v>41</v>
-      </c>
       <c r="W5" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="X5" s="14" t="s">
-        <v>119</v>
+        <v>18</v>
+      </c>
+      <c r="X5" s="15" t="s">
+        <v>56</v>
       </c>
       <c r="Y5" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="Z5" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="AA5" s="15" t="s">
-        <v>96</v>
+        <v>94</v>
+      </c>
+      <c r="Z5" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA5" s="14" t="s">
+        <v>2</v>
       </c>
       <c r="AB5" s="14" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="AC5" s="14" t="s">
-        <v>2</v>
+        <v>104</v>
       </c>
       <c r="AD5" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="AE5" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="AF5" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="AG5" s="16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:33" s="5" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="AE5" s="16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" s="5" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>163</v>
@@ -2568,366 +2499,324 @@
         <v>1</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="G6" s="19" t="s">
-        <v>137</v>
+        <v>167</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>160</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="I6" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="J6" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q6" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="X6" s="19" t="s">
-        <v>87</v>
+        <v>58</v>
+      </c>
+      <c r="O6" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="V6" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y6" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z6" s="19" t="s">
+        <v>153</v>
       </c>
       <c r="AA6" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB6" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC6" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF6" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG6" s="21" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="7" spans="1:33" s="1" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+      <c r="AD6" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE6" s="21" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B7" s="22" t="s">
         <v>162</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="O7" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="V7" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y7" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z7" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="AA7" s="24" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD7" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE7" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="G7" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="H7" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="I7" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="J7" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q7" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="X7" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA7" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB7" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC7" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF7" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG7" s="26" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" spans="1:33" s="1" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>127</v>
-      </c>
       <c r="D8" s="23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>165</v>
-      </c>
-      <c r="G8" s="24" t="s">
-        <v>137</v>
+        <v>164</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>36</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="I8" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q8" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="X8" s="24" t="s">
-        <v>87</v>
+        <v>58</v>
+      </c>
+      <c r="O8" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="V8" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y8" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z8" s="24" t="s">
+        <v>153</v>
       </c>
       <c r="AA8" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB8" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC8" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF8" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG8" s="26" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:33" s="1" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+      <c r="AD8" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE8" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B9" s="22" t="s">
         <v>43</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D9" s="23" t="s">
         <v>55</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="G9" s="24" t="s">
-        <v>137</v>
+        <v>80</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>140</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="I9" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="J9" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q9" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="X9" s="24" t="s">
-        <v>87</v>
+        <v>58</v>
+      </c>
+      <c r="O9" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="V9" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y9" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z9" s="24" t="s">
+        <v>153</v>
       </c>
       <c r="AA9" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB9" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC9" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF9" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG9" s="26" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="10" spans="1:33" s="1" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+      <c r="AD9" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE9" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="G10" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="H10" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="O10" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="V10" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y10" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z10" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="AA10" s="24" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD10" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE10" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" s="1" customFormat="1" ht="102" x14ac:dyDescent="0.2">
+      <c r="A11" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="22" t="s">
         <v>101</v>
-      </c>
-      <c r="E10" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="G10" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="H10" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="I10" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="J10" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q10" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="X10" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA10" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB10" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC10" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF10" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG10" s="26" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="11" spans="1:33" s="1" customFormat="1" ht="105.6" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>103</v>
       </c>
       <c r="C11" s="22" t="s">
         <v>50</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E11" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="F11" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="G11" s="24" t="s">
-        <v>137</v>
+      <c r="G11" s="23" t="s">
+        <v>30</v>
       </c>
       <c r="H11" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="I11" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="J11" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q11" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="X11" s="24" t="s">
-        <v>87</v>
+        <v>58</v>
+      </c>
+      <c r="O11" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="V11" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y11" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z11" s="24" t="s">
+        <v>153</v>
       </c>
       <c r="AA11" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB11" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC11" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF11" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG11" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD11" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE11" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:31" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="23" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="12" spans="1:33" s="1" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="D12" s="23" t="s">
+      <c r="E12" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="O12" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="V12" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y12" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z12" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="AA12" s="24" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE12" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:31" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A13" s="22" t="s">
         <v>90</v>
-      </c>
-      <c r="E12" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="G12" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="H12" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="I12" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="J12" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q12" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="X12" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA12" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB12" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC12" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF12" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG12" s="26" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:33" s="1" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
-        <v>92</v>
       </c>
       <c r="B13" s="22" t="s">
         <v>52</v>
@@ -2936,111 +2825,96 @@
         <v>46</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="G13" s="24" t="s">
-        <v>137</v>
+        <v>108</v>
+      </c>
+      <c r="G13" s="23" t="s">
+        <v>120</v>
       </c>
       <c r="H13" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="I13" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="J13" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q13" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="X13" s="24" t="s">
-        <v>87</v>
+        <v>58</v>
+      </c>
+      <c r="O13" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="V13" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y13" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z13" s="24" t="s">
+        <v>153</v>
       </c>
       <c r="AA13" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB13" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC13" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF13" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG13" s="26" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:33" s="1" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+      <c r="AD13" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE13" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:31" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A14" s="22" t="s">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>141</v>
+        <v>168</v>
       </c>
       <c r="D14" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="E14" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="H14" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="F14" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="G14" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="H14" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="J14" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q14" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="X14" s="24" t="s">
-        <v>87</v>
+      <c r="O14" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="V14" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y14" s="24" t="s">
+        <v>58</v>
       </c>
       <c r="Z14" s="24" t="s">
-        <v>59</v>
+        <v>153</v>
       </c>
       <c r="AA14" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB14" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC14" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF14" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AG14" s="26" t="s">
-        <v>88</v>
+        <v>135</v>
+      </c>
+      <c r="AD14" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE14" s="26" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A2:AF2"/>
-    <mergeCell ref="J4:P4"/>
-    <mergeCell ref="Q4:W4"/>
-    <mergeCell ref="Y4:AA4"/>
-    <mergeCell ref="AF4:AG4"/>
+    <mergeCell ref="A2:AD2"/>
+    <mergeCell ref="H4:N4"/>
+    <mergeCell ref="O4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="AD4:AE4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -3050,35 +2924,35 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J42"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" style="27" customWidth="1"/>
-    <col min="4" max="4" width="79.44140625" style="23" customWidth="1"/>
-    <col min="5" max="5" width="34.109375" style="28" customWidth="1"/>
-    <col min="6" max="6" width="35.6640625" style="28" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" style="27" customWidth="1"/>
+    <col min="4" max="4" width="79.42578125" style="23" customWidth="1"/>
+    <col min="5" max="5" width="34.140625" style="28" customWidth="1"/>
+    <col min="6" max="6" width="35.7109375" style="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="69" t="s">
-        <v>79</v>
-      </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
+    <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A2" s="73" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
       <c r="I2" s="29"/>
       <c r="J2" s="29"/>
     </row>
-    <row r="3" spans="1:10" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="B3" s="6"/>
       <c r="C3" s="30"/>
       <c r="D3" s="31"/>
@@ -3089,128 +2963,128 @@
       <c r="I3" s="6"/>
       <c r="J3" s="6"/>
     </row>
-    <row r="4" spans="1:10" s="5" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" s="5" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="B4" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="92" t="s">
-        <v>131</v>
-      </c>
-      <c r="D4" s="93"/>
+        <v>103</v>
+      </c>
+      <c r="C4" s="96" t="s">
+        <v>129</v>
+      </c>
+      <c r="D4" s="97"/>
       <c r="E4" s="34" t="s">
         <v>157</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="91" t="s">
-        <v>77</v>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="95" t="s">
+        <v>75</v>
       </c>
       <c r="B5" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="83" t="s">
-        <v>97</v>
-      </c>
-      <c r="D5" s="84"/>
+      <c r="C5" s="87" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="88"/>
       <c r="E5" s="36" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="91"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="95"/>
       <c r="B6" s="35" t="s">
         <v>158</v>
       </c>
-      <c r="C6" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D6" s="84"/>
+      <c r="C6" s="87" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="88"/>
       <c r="E6" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F6" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="91"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="95"/>
       <c r="B7" s="35" t="s">
-        <v>136</v>
-      </c>
-      <c r="C7" s="83" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="84"/>
+        <v>134</v>
+      </c>
+      <c r="C7" s="87" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="88"/>
       <c r="E7" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F7" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="91"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="95"/>
       <c r="B8" s="40" t="s">
-        <v>94</v>
-      </c>
-      <c r="C8" s="85" t="s">
-        <v>146</v>
-      </c>
-      <c r="D8" s="86"/>
+        <v>92</v>
+      </c>
+      <c r="C8" s="89" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" s="90"/>
       <c r="E8" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="53.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="91"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" s="1" customFormat="1" ht="53.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="95"/>
       <c r="B9" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="85" t="s">
-        <v>151</v>
-      </c>
-      <c r="D9" s="86"/>
+      <c r="C9" s="89" t="s">
+        <v>149</v>
+      </c>
+      <c r="D9" s="90"/>
       <c r="E9" s="41" t="s">
         <v>49</v>
       </c>
       <c r="F9" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="91"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="95"/>
       <c r="B10" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C10" s="87" t="s">
-        <v>91</v>
-      </c>
-      <c r="D10" s="90"/>
+        <v>114</v>
+      </c>
+      <c r="C10" s="91" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="94"/>
       <c r="E10" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F10" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="91"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="95"/>
       <c r="B11" s="35" t="s">
-        <v>147</v>
-      </c>
-      <c r="C11" s="87" t="s">
         <v>144</v>
       </c>
-      <c r="D11" s="88"/>
+      <c r="C11" s="91" t="s">
+        <v>142</v>
+      </c>
+      <c r="D11" s="92"/>
       <c r="E11" s="41" t="s">
         <v>49</v>
       </c>
@@ -3218,415 +3092,415 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:10" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="91"/>
+    <row r="12" spans="1:10" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="95"/>
       <c r="B12" s="35" t="s">
-        <v>128</v>
-      </c>
-      <c r="C12" s="87" t="s">
-        <v>76</v>
-      </c>
-      <c r="D12" s="90"/>
+        <v>126</v>
+      </c>
+      <c r="C12" s="91" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="94"/>
       <c r="E12" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F12" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="91"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="95"/>
       <c r="B13" s="40" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13" s="91" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="94"/>
+      <c r="E13" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="C13" s="87" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="90"/>
-      <c r="E13" s="38" t="s">
-        <v>135</v>
-      </c>
       <c r="F13" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" s="1" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="91"/>
-      <c r="B14" s="78" t="s">
-        <v>100</v>
-      </c>
-      <c r="C14" s="81" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="82"/>
-      <c r="E14" s="104" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="1" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="95"/>
+      <c r="B14" s="82" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="86"/>
+      <c r="E14" s="108" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="107" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="91"/>
-      <c r="B15" s="79"/>
+      <c r="F14" s="111" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="95"/>
+      <c r="B15" s="83"/>
       <c r="C15" s="42" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="E15" s="105"/>
-      <c r="F15" s="108"/>
-    </row>
-    <row r="16" spans="1:10" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="91"/>
-      <c r="B16" s="79"/>
+        <v>127</v>
+      </c>
+      <c r="E15" s="109"/>
+      <c r="F15" s="112"/>
+    </row>
+    <row r="16" spans="1:10" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="95"/>
+      <c r="B16" s="83"/>
       <c r="C16" s="42" t="s">
         <v>42</v>
       </c>
       <c r="D16" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="105"/>
-      <c r="F16" s="108"/>
-    </row>
-    <row r="17" spans="1:6" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="91"/>
-      <c r="B17" s="79"/>
+      <c r="E16" s="109"/>
+      <c r="F16" s="112"/>
+    </row>
+    <row r="17" spans="1:6" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="95"/>
+      <c r="B17" s="83"/>
       <c r="C17" s="42" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D17" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="E17" s="105"/>
-      <c r="F17" s="108"/>
-    </row>
-    <row r="18" spans="1:6" s="1" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="91"/>
-      <c r="B18" s="79"/>
+      <c r="E17" s="109"/>
+      <c r="F17" s="112"/>
+    </row>
+    <row r="18" spans="1:6" s="1" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="95"/>
+      <c r="B18" s="83"/>
       <c r="C18" s="42" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>112</v>
-      </c>
-      <c r="E18" s="105"/>
-      <c r="F18" s="108"/>
-    </row>
-    <row r="19" spans="1:6" s="1" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="91"/>
-      <c r="B19" s="79"/>
+        <v>110</v>
+      </c>
+      <c r="E18" s="109"/>
+      <c r="F18" s="112"/>
+    </row>
+    <row r="19" spans="1:6" s="1" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="95"/>
+      <c r="B19" s="83"/>
       <c r="C19" s="42" t="s">
         <v>169</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="E19" s="105"/>
-      <c r="F19" s="108"/>
-    </row>
-    <row r="20" spans="1:6" s="1" customFormat="1" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="91"/>
-      <c r="B20" s="79"/>
+        <v>112</v>
+      </c>
+      <c r="E19" s="109"/>
+      <c r="F19" s="112"/>
+    </row>
+    <row r="20" spans="1:6" s="1" customFormat="1" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="95"/>
+      <c r="B20" s="83"/>
       <c r="C20" s="42" t="s">
         <v>44</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="E20" s="105"/>
-      <c r="F20" s="108"/>
-    </row>
-    <row r="21" spans="1:6" s="1" customFormat="1" ht="57.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="91"/>
-      <c r="B21" s="80"/>
+        <v>154</v>
+      </c>
+      <c r="E20" s="109"/>
+      <c r="F20" s="112"/>
+    </row>
+    <row r="21" spans="1:6" s="1" customFormat="1" ht="57.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="95"/>
+      <c r="B21" s="84"/>
       <c r="C21" s="42" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="E21" s="106"/>
-      <c r="F21" s="109"/>
-    </row>
-    <row r="22" spans="1:6" s="1" customFormat="1" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="91"/>
-      <c r="B22" s="89" t="s">
-        <v>142</v>
-      </c>
-      <c r="C22" s="97" t="s">
-        <v>71</v>
-      </c>
-      <c r="D22" s="98"/>
-      <c r="E22" s="104" t="s">
+        <v>128</v>
+      </c>
+      <c r="E21" s="110"/>
+      <c r="F21" s="113"/>
+    </row>
+    <row r="22" spans="1:6" s="1" customFormat="1" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="95"/>
+      <c r="B22" s="93" t="s">
+        <v>139</v>
+      </c>
+      <c r="C22" s="101" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" s="102"/>
+      <c r="E22" s="108" t="s">
         <v>49</v>
       </c>
-      <c r="F22" s="107" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="91"/>
-      <c r="B23" s="79"/>
+      <c r="F22" s="111" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="95"/>
+      <c r="B23" s="83"/>
       <c r="C23" s="43" t="s">
+        <v>150</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="E23" s="109"/>
+      <c r="F23" s="112"/>
+    </row>
+    <row r="24" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="95"/>
+      <c r="B24" s="83"/>
+      <c r="C24" s="43" t="s">
+        <v>148</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24" s="109"/>
+      <c r="F24" s="112"/>
+    </row>
+    <row r="25" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="95"/>
+      <c r="B25" s="83"/>
+      <c r="C25" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="E25" s="109"/>
+      <c r="F25" s="112"/>
+    </row>
+    <row r="26" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="95"/>
+      <c r="B26" s="83"/>
+      <c r="C26" s="43" t="s">
         <v>152</v>
       </c>
-      <c r="D23" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="E23" s="105"/>
-      <c r="F23" s="108"/>
-    </row>
-    <row r="24" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="91"/>
-      <c r="B24" s="79"/>
-      <c r="C24" s="43" t="s">
-        <v>150</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="E24" s="105"/>
-      <c r="F24" s="108"/>
-    </row>
-    <row r="25" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="91"/>
-      <c r="B25" s="79"/>
-      <c r="C25" s="43" t="s">
-        <v>115</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="E25" s="105"/>
-      <c r="F25" s="108"/>
-    </row>
-    <row r="26" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="91"/>
-      <c r="B26" s="79"/>
-      <c r="C26" s="43" t="s">
-        <v>154</v>
-      </c>
       <c r="D26" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="E26" s="105"/>
-      <c r="F26" s="108"/>
-    </row>
-    <row r="27" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="91"/>
-      <c r="B27" s="79"/>
+        <v>35</v>
+      </c>
+      <c r="E26" s="109"/>
+      <c r="F26" s="112"/>
+    </row>
+    <row r="27" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="95"/>
+      <c r="B27" s="83"/>
       <c r="C27" s="43" t="s">
         <v>170</v>
       </c>
       <c r="D27" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="E27" s="105"/>
-      <c r="F27" s="108"/>
-    </row>
-    <row r="28" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="91"/>
-      <c r="B28" s="79"/>
+        <v>116</v>
+      </c>
+      <c r="E27" s="109"/>
+      <c r="F27" s="112"/>
+    </row>
+    <row r="28" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="95"/>
+      <c r="B28" s="83"/>
       <c r="C28" s="43" t="s">
         <v>41</v>
       </c>
       <c r="D28" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="E28" s="105"/>
-      <c r="F28" s="108"/>
-    </row>
-    <row r="29" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="91"/>
-      <c r="B29" s="80"/>
+      <c r="E28" s="109"/>
+      <c r="F28" s="112"/>
+    </row>
+    <row r="29" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="95"/>
+      <c r="B29" s="84"/>
       <c r="C29" s="45" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D29" s="46" t="s">
-        <v>109</v>
-      </c>
-      <c r="E29" s="106"/>
-      <c r="F29" s="109"/>
-    </row>
-    <row r="30" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="91"/>
+        <v>106</v>
+      </c>
+      <c r="E29" s="110"/>
+      <c r="F29" s="113"/>
+    </row>
+    <row r="30" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="95"/>
       <c r="B30" s="47" t="s">
-        <v>119</v>
-      </c>
-      <c r="C30" s="99" t="s">
-        <v>153</v>
-      </c>
-      <c r="D30" s="100"/>
+        <v>117</v>
+      </c>
+      <c r="C30" s="103" t="s">
+        <v>151</v>
+      </c>
+      <c r="D30" s="104"/>
       <c r="E30" s="41" t="s">
         <v>49</v>
       </c>
       <c r="F30" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="91"/>
-      <c r="B31" s="75" t="s">
-        <v>63</v>
-      </c>
-      <c r="C31" s="87" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="90"/>
-      <c r="E31" s="104" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="95"/>
+      <c r="B31" s="79" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" s="91" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="94"/>
+      <c r="E31" s="108" t="s">
         <v>49</v>
       </c>
-      <c r="F31" s="107" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="91"/>
-      <c r="B32" s="76"/>
+      <c r="F31" s="111" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="95"/>
+      <c r="B32" s="80"/>
       <c r="C32" s="48" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D32" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="E32" s="105"/>
-      <c r="F32" s="108"/>
-    </row>
-    <row r="33" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="91"/>
-      <c r="B33" s="76"/>
+        <v>17</v>
+      </c>
+      <c r="E32" s="109"/>
+      <c r="F32" s="112"/>
+    </row>
+    <row r="33" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="95"/>
+      <c r="B33" s="80"/>
       <c r="C33" s="48" t="s">
         <v>56</v>
       </c>
       <c r="D33" s="50" t="s">
-        <v>149</v>
-      </c>
-      <c r="E33" s="105"/>
-      <c r="F33" s="108"/>
-    </row>
-    <row r="34" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="91"/>
-      <c r="B34" s="77"/>
+        <v>147</v>
+      </c>
+      <c r="E33" s="109"/>
+      <c r="F33" s="112"/>
+    </row>
+    <row r="34" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="95"/>
+      <c r="B34" s="81"/>
       <c r="C34" s="48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D34" s="50" t="s">
-        <v>65</v>
-      </c>
-      <c r="E34" s="106"/>
-      <c r="F34" s="109"/>
-    </row>
-    <row r="35" spans="1:6" s="1" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="94" t="s">
-        <v>78</v>
+        <v>64</v>
+      </c>
+      <c r="E34" s="110"/>
+      <c r="F34" s="113"/>
+    </row>
+    <row r="35" spans="1:6" s="1" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="98" t="s">
+        <v>76</v>
       </c>
       <c r="B35" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="C35" s="87" t="s">
-        <v>86</v>
-      </c>
-      <c r="D35" s="90"/>
+        <v>93</v>
+      </c>
+      <c r="C35" s="91" t="s">
+        <v>84</v>
+      </c>
+      <c r="D35" s="94"/>
       <c r="E35" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F35" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" s="1" customFormat="1" ht="21.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="94"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="98"/>
       <c r="B36" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="C36" s="87" t="s">
-        <v>37</v>
-      </c>
-      <c r="D36" s="90"/>
+      <c r="C36" s="91" t="s">
+        <v>38</v>
+      </c>
+      <c r="D36" s="94"/>
       <c r="E36" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F36" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" s="1" customFormat="1" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="94"/>
-      <c r="B37" s="75" t="s">
-        <v>33</v>
-      </c>
-      <c r="C37" s="95" t="s">
-        <v>121</v>
-      </c>
-      <c r="D37" s="96"/>
-      <c r="E37" s="101" t="s">
-        <v>135</v>
-      </c>
-      <c r="F37" s="107" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="94"/>
-      <c r="B38" s="76"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="98"/>
+      <c r="B37" s="79" t="s">
+        <v>34</v>
+      </c>
+      <c r="C37" s="99" t="s">
+        <v>119</v>
+      </c>
+      <c r="D37" s="100"/>
+      <c r="E37" s="105" t="s">
+        <v>133</v>
+      </c>
+      <c r="F37" s="111" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="98"/>
+      <c r="B38" s="80"/>
       <c r="C38" s="43" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D38" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="102"/>
-      <c r="F38" s="108"/>
-    </row>
-    <row r="39" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="94"/>
-      <c r="B39" s="76"/>
+      <c r="E38" s="106"/>
+      <c r="F38" s="112"/>
+    </row>
+    <row r="39" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="98"/>
+      <c r="B39" s="80"/>
       <c r="C39" s="43" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>70</v>
-      </c>
-      <c r="E39" s="102"/>
-      <c r="F39" s="108"/>
-    </row>
-    <row r="40" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="94"/>
-      <c r="B40" s="76"/>
+        <v>69</v>
+      </c>
+      <c r="E39" s="106"/>
+      <c r="F39" s="112"/>
+    </row>
+    <row r="40" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="98"/>
+      <c r="B40" s="80"/>
       <c r="C40" s="43" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D40" s="44" t="s">
-        <v>98</v>
-      </c>
-      <c r="E40" s="102"/>
-      <c r="F40" s="108"/>
-    </row>
-    <row r="41" spans="1:6" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A41" s="94"/>
-      <c r="B41" s="76"/>
+        <v>96</v>
+      </c>
+      <c r="E40" s="106"/>
+      <c r="F40" s="112"/>
+    </row>
+    <row r="41" spans="1:6" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A41" s="98"/>
+      <c r="B41" s="80"/>
       <c r="C41" s="43" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D41" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="E41" s="102"/>
-      <c r="F41" s="108"/>
-    </row>
-    <row r="42" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="94"/>
-      <c r="B42" s="77"/>
+      <c r="E41" s="106"/>
+      <c r="F41" s="112"/>
+    </row>
+    <row r="42" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="98"/>
+      <c r="B42" s="81"/>
       <c r="C42" s="51" t="s">
         <v>57</v>
       </c>
       <c r="D42" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E42" s="103"/>
-      <c r="F42" s="110"/>
+      <c r="E42" s="107"/>
+      <c r="F42" s="114"/>
     </row>
   </sheetData>
   <mergeCells count="32">
@@ -3670,43 +3544,43 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" style="10" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="54.44140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="54.42578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="111" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="111"/>
-      <c r="C3" s="111"/>
-      <c r="D3" s="112"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="113"/>
-      <c r="B4" s="113"/>
-      <c r="C4" s="113"/>
-      <c r="D4" s="114"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="115"/>
-      <c r="B5" s="115"/>
-      <c r="C5" s="115"/>
-      <c r="D5" s="116"/>
-    </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="115" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="115"/>
+      <c r="C3" s="115"/>
+      <c r="D3" s="116"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="117"/>
+      <c r="B4" s="117"/>
+      <c r="C4" s="117"/>
+      <c r="D4" s="118"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="119"/>
+      <c r="B5" s="119"/>
+      <c r="C5" s="119"/>
+      <c r="D5" s="120"/>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A6" s="52" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" s="52" t="s">
         <v>159</v>
@@ -3715,56 +3589,56 @@
         <v>45</v>
       </c>
       <c r="D6" s="52" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="53"/>
       <c r="B7" s="54"/>
       <c r="C7" s="55"/>
       <c r="D7" s="53"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="53"/>
       <c r="B8" s="54"/>
       <c r="C8" s="55"/>
       <c r="D8" s="53"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="53"/>
       <c r="B9" s="54"/>
       <c r="C9" s="55"/>
       <c r="D9" s="53"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="53"/>
       <c r="B10" s="54"/>
       <c r="C10" s="55"/>
       <c r="D10" s="53"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="111" t="s">
-        <v>126</v>
-      </c>
-      <c r="B15" s="111"/>
-      <c r="C15" s="111"/>
-      <c r="D15" s="112"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="113"/>
-      <c r="B16" s="113"/>
-      <c r="C16" s="113"/>
-      <c r="D16" s="114"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="115"/>
-      <c r="B17" s="115"/>
-      <c r="C17" s="115"/>
-      <c r="D17" s="116"/>
-    </row>
-    <row r="18" spans="1:4" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="115" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" s="115"/>
+      <c r="C15" s="115"/>
+      <c r="D15" s="116"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="117"/>
+      <c r="B16" s="117"/>
+      <c r="C16" s="117"/>
+      <c r="D16" s="118"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="119"/>
+      <c r="B17" s="119"/>
+      <c r="C17" s="119"/>
+      <c r="D17" s="120"/>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A18" s="52" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" s="52" t="s">
         <v>159</v>
@@ -3773,52 +3647,52 @@
         <v>45</v>
       </c>
       <c r="D18" s="52" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="53" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B19" s="54" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="55">
         <v>43343</v>
       </c>
       <c r="D19" s="53" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A20" s="53" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B20" s="54" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C20" s="55">
         <v>43396</v>
       </c>
       <c r="D20" s="53" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="132" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A21" s="53" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B21" s="54" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C21" s="55">
         <v>43413</v>
       </c>
       <c r="D21" s="53" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A22" s="53" t="s">
         <v>173</v>
       </c>
@@ -3830,6 +3704,20 @@
       </c>
       <c r="D22" s="53" t="s">
         <v>175</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A23" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="B23" s="54" t="s">
+        <v>176</v>
+      </c>
+      <c r="C23" s="55">
+        <v>43664</v>
+      </c>
+      <c r="D23" s="53" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs - Test and SA reports
Signed-off-by: Prasad Jondhale <prasad.jondhale@ti.com>
</commit_message>
<xml_diff>
--- a/docs/test_report/ethfw_testreport.xlsx
+++ b/docs/test_report/ethfw_testreport.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="12840" yWindow="0" windowWidth="13725" windowHeight="8355" tabRatio="599"/>
+    <workbookView xWindow="-15" yWindow="0" windowWidth="12300" windowHeight="11085" tabRatio="599" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Revision History" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Details'!$A$5:$AD$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Details'!$A$5:$AF$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Revision History'!#REF!</definedName>
     <definedName name="Test_Category">Help!#REF!</definedName>
   </definedNames>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="268">
   <si>
     <t>Test is not required for this release (e.g., test case not supported for targeted platform)</t>
   </si>
@@ -30,15 +30,33 @@
     <t>ETHFW-58 : [EthFW][OS]OSAL:EMAC Osal:Baremetal implementation of EMAL osal interface should be integrated into the switch firmware</t>
   </si>
   <si>
+    <t xml:space="preserve">[EthFW][Performance]Switching Performance:Head of line blocking test </t>
+  </si>
+  <si>
+    <t>OS:emac_lld should be validated on  lock step variant of TI RTOS config also</t>
+  </si>
+  <si>
+    <t>[EthFW][Packaging] The ethernet firmware shall be hosted in a separate repo to support firmware only release decoupled from rest of Processor SDK</t>
+  </si>
+  <si>
     <t>IR</t>
   </si>
   <si>
+    <t>IPC:Support for switch configuration from remote core</t>
+  </si>
+  <si>
+    <t>Wire rate switching  for all frame sizes with VLAN stripping should be under acceptable criteria</t>
+  </si>
+  <si>
     <t>Summary</t>
   </si>
   <si>
     <t>TI Information - Selective Disclosure</t>
   </si>
   <si>
+    <t>ETHFW-491</t>
+  </si>
+  <si>
     <t>Test Case covers usability/api/look and feel aspects of the module including out-of box (OOB) experience</t>
   </si>
   <si>
@@ -51,6 +69,9 @@
     <t>Author</t>
   </si>
   <si>
+    <t>[EthFw][IPC]IPC: All cores must allocate cores own MAC Address/IP address by sending msg to central IP/MAC resource manager running on master core</t>
+  </si>
+  <si>
     <t>PASS</t>
   </si>
   <si>
@@ -75,12 +96,24 @@
     <t>A description of the pass and fail criteria for the test case</t>
   </si>
   <si>
+    <t>ETHFW-490</t>
+  </si>
+  <si>
+    <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN (no packet modification)</t>
+  </si>
+  <si>
+    <t>ETHFW-55 : [EthFW][OS]OS:cpsw_lld should be validated on  lock step variant of TI RTOS config</t>
+  </si>
+  <si>
     <t>This Test case is identified to run for Sanity Checks. These are mainly the basic tests that need to be run as part of entry to validate phase</t>
   </si>
   <si>
     <t>Sanity</t>
   </si>
   <si>
+    <t>ETHFW-76 : [EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN stripping</t>
+  </si>
+  <si>
     <t>ETHFW-160</t>
   </si>
   <si>
@@ -105,24 +138,39 @@
     <t>ETHFW-385</t>
   </si>
   <si>
+    <t>10/18/2019</t>
+  </si>
+  <si>
     <t>Test cases derived by division of inputs and outputs ranges to ensure a representative test value can be selected for each class or range.</t>
   </si>
   <si>
+    <t>26</t>
+  </si>
+  <si>
     <t xml:space="preserve">The test plan is expected to leverage various types of testing methods to demonstrate software meets expectations.  This field identifies the type of test method associated with the test case.  The types of tests are described below: </t>
   </si>
   <si>
     <t>EthFW OS Test - CPSW LLD validation</t>
   </si>
   <si>
+    <t>Wire rate switching  for all frame sizes with VLAN insertion should be under acceptable criteria</t>
+  </si>
+  <si>
     <t>Confirm packet interrupts occur at periodic 500us interval only when interrupt pacing is enabled. The interrupt pacing is triggered by TImer interrupt</t>
   </si>
   <si>
+    <t>[EthFw][IPC]IPC: Integration with linux virtual driver running on A72 remote core</t>
+  </si>
+  <si>
     <t>EthFW EMAC OSAL Test - Baremetal implementation</t>
   </si>
   <si>
     <t>100 %</t>
   </si>
   <si>
+    <t>Should able to run application successfully</t>
+  </si>
+  <si>
     <t>EthFW System Test - PMU Driver Integration</t>
   </si>
   <si>
@@ -141,18 +189,33 @@
     <t>This field provides necessary JIRA bug ID for any failed test cases.</t>
   </si>
   <si>
+    <t>ETHFW-74 : [EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN (no packet modification)</t>
+  </si>
+  <si>
     <t>ETHFW-37 : [EthFW][System]Driver Integration:UART: UART driver should be integrated and used for development time log prints</t>
   </si>
   <si>
     <t>Test Blocked because of other test case failure, an Open MR from previous Release, feature not implemented yet, feature not supported by hardware</t>
   </si>
   <si>
+    <t>ETHFW-497</t>
+  </si>
+  <si>
     <t>Failure Mode Analysis</t>
   </si>
   <si>
+    <t>ETHFW-493</t>
+  </si>
+  <si>
     <t>Interface</t>
   </si>
   <si>
+    <t>ETHFW-494</t>
+  </si>
+  <si>
+    <t>ETHFW-77 : [EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port</t>
+  </si>
+  <si>
     <t>EthFW OS Test - TI RTOS integration</t>
   </si>
   <si>
@@ -165,6 +228,9 @@
     <t>ETHFW-163</t>
   </si>
   <si>
+    <t>[EthFw][IPC]IPC:Remote core invocation APIs for switch config should be stateless on remote core side</t>
+  </si>
+  <si>
     <t>Should be able to get PMU counters for perfomance profiling</t>
   </si>
   <si>
@@ -177,12 +243,21 @@
     <t>ETHFW-161</t>
   </si>
   <si>
+    <t>ETHFW-48 : [EthFw][IPC]IPC: Initial handshake and CPSW init completion notification</t>
+  </si>
+  <si>
     <t>Test Plan Name</t>
   </si>
   <si>
     <t>EthFW System Test - UART Driver Integration</t>
   </si>
   <si>
+    <t>HOL (head of line) blocking doesnt exist in switching</t>
+  </si>
+  <si>
+    <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN (no packet modification)</t>
+  </si>
+  <si>
     <t>Tests covering aspects related to the software interfaces including range checking of interface variable</t>
   </si>
   <si>
@@ -192,21 +267,41 @@
     <t>ETHFW-54 : [EthFW][OS]OS:TI RTOS: TI RTOS should be integrated into the switch firmware</t>
   </si>
   <si>
+    <t>ETHFW-53 : [EthFw][IPC]IPC: Integration with CPSW LLD RTOS driver running on A72/MCU_SS R5F remote core</t>
+  </si>
+  <si>
     <t>Regression</t>
   </si>
   <si>
     <t>NRQ</t>
   </si>
   <si>
+    <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port</t>
+  </si>
+  <si>
+    <t>The ethernet firmware shall be hosted in a separate repo to support firmware only release decoupled from rest of Processor SDK
+This will require ethernet firmware to have independent release plan (and version plan) decoupled from Processor SDK PDK
+This is needed to allow LCPD to consume CPSW Ethernet switch firmware without waiting for Processor SDK RTOS</t>
+  </si>
+  <si>
+    <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN stripping</t>
+  </si>
+  <si>
     <t>X</t>
   </si>
   <si>
     <t>Requirement/ Design/ Architecture ID</t>
   </si>
   <si>
+    <t>Should able to configure Switch from all cores</t>
+  </si>
+  <si>
     <t>Unit</t>
   </si>
   <si>
+    <t>ETHFW-44 : [EthFw][IPC]IPC:Remote core invocation APIs for switch config should be stateless on remote core side</t>
+  </si>
+  <si>
     <t>[EthFW][System]Driver Integration:GPTIMER: GPTIMER driver should be integrated</t>
   </si>
   <si>
@@ -219,6 +314,9 @@
     <t>This Test case is identified to run as part of the full release cycle</t>
   </si>
   <si>
+    <t>ETHFW-78 : [EthFW][Performance]Switching Performance:Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8</t>
+  </si>
+  <si>
     <t>Revision History</t>
   </si>
   <si>
@@ -234,9 +332,18 @@
     <t>Test Passed</t>
   </si>
   <si>
+    <t>ETHFW-502</t>
+  </si>
+  <si>
     <t>As part of test planning, various methods are used to derive test cases.  This field identifies the test derivation method was associated with this test case.  The possible derivation methods are defined below:</t>
   </si>
   <si>
+    <t>All core must register them self by sending msg to master core</t>
+  </si>
+  <si>
+    <t>[EthFW][Performance]Switching Performance:Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8</t>
+  </si>
+  <si>
     <t>J7-EVM</t>
   </si>
   <si>
@@ -249,16 +356,37 @@
     <t>Reference to the required test hardware set-up and environment</t>
   </si>
   <si>
+    <t>ETHFW-489</t>
+  </si>
+  <si>
     <t>Test Plan Information</t>
   </si>
   <si>
     <t>Test Report Information</t>
   </si>
   <si>
+    <t>Ethernet Firmware IPC should be integrated with linux virtual netdev driver running on A72 remote core</t>
+  </si>
+  <si>
     <t>Test Plan Template Help</t>
   </si>
   <si>
+    <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port</t>
+  </si>
+  <si>
+    <t>ETHFW-496</t>
+  </si>
+  <si>
     <t>ETHFW-39 : [EthFW][System]Driver Integration:GPTIMER: GPTIMER driver should be integrated</t>
+  </si>
+  <si>
+    <t>[EthFW][Performance]Switching Performance:Wire rate broadcast/Multicast traffic</t>
+  </si>
+  <si>
+    <t>For generic kernel driver in mainline dependency on pre-initialization is not good experience (people use different bootloader boot sequence etc). So there should be a way to query of firmware is loaded and if not let driver load it from filesystem.</t>
+  </si>
+  <si>
+    <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN insertion</t>
   </si>
   <si>
     <t>[EthFW][System]Driver Integration:TISCI: TISCI client driver should be integrated for DMSC IPC</t>
@@ -273,12 +401,21 @@
 -- Added project level detail information to summary page (e.g., product name, version, report date, Platform, OS)</t>
   </si>
   <si>
+    <t>[EthFw][IPC]IPC:Support for switch configuration from remote core</t>
+  </si>
+  <si>
+    <t>ETHFW-79 : [EthFW][Performance]Switching Performance:Wire rate broadcast/Multicast traffic</t>
+  </si>
+  <si>
     <t>Unique Test Case name</t>
   </si>
   <si>
     <t>[EthFW][System]Driver Integration:PMU: PMU driver should be integrated</t>
   </si>
   <si>
+    <t>ETHFW-507</t>
+  </si>
+  <si>
     <t>Software build name/information for which the test results apply</t>
   </si>
   <si>
@@ -294,21 +431,39 @@
     <t>ETHFW-38 : [EthFW][System]Driver Integration:PMU: PMU driver should be integrated</t>
   </si>
   <si>
+    <t>Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port should be under acceptable criteria</t>
+  </si>
+  <si>
+    <t>Switching Performance:Wire rate switching  for all frame sizes without VLAN.</t>
+  </si>
+  <si>
     <t>Detailed description of the test and steps required</t>
   </si>
   <si>
     <t>ETHFW-177</t>
   </si>
   <si>
+    <t>ETHFW-73 : [EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes without VLAN.</t>
+  </si>
+  <si>
     <t>QRAS AP00216 automotive and functional safety</t>
   </si>
   <si>
     <t>Requirement ID (or Design ID or Architecture ID)</t>
   </si>
   <si>
+    <t>ETHFW-499</t>
+  </si>
+  <si>
     <t>Build Name</t>
   </si>
   <si>
+    <t>ETHFW-75 : [EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN insertion</t>
+  </si>
+  <si>
+    <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN stripping</t>
+  </si>
+  <si>
     <t>Full</t>
   </si>
   <si>
@@ -333,7 +488,18 @@
     <t>EthFW System Test - GPTIMER Driver Integration</t>
   </si>
   <si>
+    <t xml:space="preserve">ETHFW-80 : [EthFW][Performance]Switching Performance:Head of line blocking test </t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
     <t>B</t>
+  </si>
+  <si>
+    <t>IPC: Sync mechanism
+  Initial shared memory based handshake
+  Notification to remote cores on CPSW initial configuration completion</t>
   </si>
   <si>
     <t>Test Matrix Field</t>
@@ -346,6 +512,9 @@
     <t>Confirm successful execution with DMSC firmware</t>
   </si>
   <si>
+    <t>ETHFW-506</t>
+  </si>
+  <si>
     <t>Test cases established based on lessons learned and expert judgement to determine situations that may cause software failures or errors to appear</t>
   </si>
   <si>
@@ -362,27 +531,48 @@
   </si>
   <si>
     <t>Initial version</t>
+  </si>
+  <si>
+    <t>ETHFW-52 : [EthFw][IPC]IPC: Integration with linux virtual driver running on A72 remote core</t>
+  </si>
+  <si>
+    <t>Wire rate switching  for all frame sizes with VLAN should be under acceptable criteria</t>
   </si>
   <si>
     <t>Test Case covers performance, profiling, latency etc. 
 IEEE Defn: To determine if the software can handle the anticipated amount of work in the required time</t>
   </si>
   <si>
+    <t>[EthFW][OS]OS:cpsw_lld should be validated on  lock step variant of TI RTOS config</t>
+  </si>
+  <si>
     <t>Boundary Value Analysis</t>
   </si>
   <si>
     <t>Test Description</t>
   </si>
   <si>
+    <t>Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8 (priority remapping) should be under acceptable criteria</t>
+  </si>
+  <si>
     <t>Stress</t>
   </si>
   <si>
     <t>Test cases derived to validate customer/user experience associated with usage of the software product (getting started, OOB look-and-feel, APIs, …)</t>
   </si>
   <si>
+    <t>ETHFW-47 : [EthFw][IPC]IPC: All cores must allocate cores own MAC Address/IP address by sending msg to central IP/MAC resource manager running on master core</t>
+  </si>
+  <si>
+    <t>Switching Performance:Wire rate broadcast/Multicast traffic</t>
+  </si>
+  <si>
     <t>Automated/Manual</t>
   </si>
   <si>
+    <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN insertion</t>
+  </si>
+  <si>
     <t>Pass/Fail Criteria</t>
   </si>
   <si>
@@ -395,19 +585,45 @@
     <t>Error Guessing</t>
   </si>
   <si>
-    <t>9</t>
+    <t>ETHFW-81 : [EthFW][Packaging] The ethernet firmware shall be released under TI-TFL license
+ETHFW-84 : [EthFW][Packaging] The ethernet firmware shall be hosted at external git.ti.com
+ETHFW-85 : [EthFW][Packaging] The ethernet firmware shall be hosted in a separate repo to support firmware only release decoupled from rest of Processor SDK</t>
+  </si>
+  <si>
+    <t>Qualification</t>
   </si>
   <si>
     <t>ETHFW-57 : [EthFW][OS]OSAL:EMAC Osal: TI RTOS implementation of EMAL osal interface should be integrated into the switch firmware</t>
   </si>
   <si>
+    <t>Switching Performance:Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8 (priority remapping)</t>
+  </si>
+  <si>
+    <t>IPC: All cores must allocate cores own MAC Address/IP address by sending msg to central IP/MAC resource manager running on master core</t>
+  </si>
+  <si>
+    <t>IPC:Remote core invocation APIs for switch config should be stateless on remote core side</t>
+  </si>
+  <si>
+    <t>Wire rate switching  for all frame sizes without VLAN should be under acceptable criteria</t>
+  </si>
+  <si>
     <t>Template Revision History</t>
   </si>
   <si>
+    <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes without VLAN.</t>
+  </si>
+  <si>
+    <t>After successfully CPSW initialization notification send to all remote cores</t>
+  </si>
+  <si>
     <t>ETHFW-158</t>
   </si>
   <si>
     <t>Test Set-up</t>
+  </si>
+  <si>
+    <t>ETHFW-505</t>
   </si>
   <si>
     <t>Tests covering functional requirements-based  aspects of the software</t>
@@ -420,6 +636,9 @@
     <t>Description</t>
   </si>
   <si>
+    <t>ETHFW-500</t>
+  </si>
+  <si>
     <t>Frank Fruth</t>
   </si>
   <si>
@@ -451,6 +670,12 @@
     <t>Test Derivation Method</t>
   </si>
   <si>
+    <t>ETHFW-503</t>
+  </si>
+  <si>
+    <t>[EthFw][IPC]IPC: Initial handshake and CPSW init completion notification</t>
+  </si>
+  <si>
     <t>Successful execution of EThFw switching test with sysbios</t>
   </si>
   <si>
@@ -460,15 +685,38 @@
     <t>Optional project-specific field that can be used to further classify specifc test area or module</t>
   </si>
   <si>
+    <t>ETHFW-43 : [EthFw][IPC]IPC:Support for switch configuration from remote core</t>
+  </si>
+  <si>
+    <t>Perform multicast and unicast tests to confirm HOL (head of line) blocking doesnt exist in switching</t>
+  </si>
+  <si>
+    <t>1. separate package for ethfw
+2. should be available at external git.ti.com
+3. should be released under TI-TFL license</t>
+  </si>
+  <si>
     <t>Functional Requirement ID(s) from the SPS that this test case covers (comma separated).  For automotive and functional safety, this may also include design ID and/or architecture IDs as well.</t>
   </si>
   <si>
+    <t>ETHFW-492</t>
+  </si>
+  <si>
+    <t>ETHFW-498</t>
+  </si>
+  <si>
     <t>Test Area</t>
   </si>
   <si>
     <t>Should successfully execute CPsw Switching App with Cpsw library linked with tirtos osal implementation</t>
   </si>
   <si>
+    <t>Wire rate broadcast/Multicast traffic should be under acceptable criteria</t>
+  </si>
+  <si>
+    <t>ETHFW-504</t>
+  </si>
+  <si>
     <t>Should able to send/receive packets through TCP/UDP/ICMP/IP</t>
   </si>
   <si>
@@ -476,6 +724,9 @@
   </si>
   <si>
     <t>Generation and Analysis of Equivalence Classes</t>
+  </si>
+  <si>
+    <t>client side application does not aware of state</t>
   </si>
   <si>
     <t>Identifies test case scope:
@@ -487,13 +738,13 @@
     <t>Requirements-Analysis</t>
   </si>
   <si>
+    <t>check in boot log remote core should able to query of firmware is loaded or not</t>
+  </si>
+  <si>
     <t>Identifies whether the case is automated or manually executed</t>
   </si>
   <si>
     <t>Use Case Analysis</t>
-  </si>
-  <si>
-    <t>ETHFW-386</t>
   </si>
   <si>
     <t>Test Case ensures that the component does not fail over time
@@ -506,21 +757,36 @@
     <t>Test cases derived from analysis of potential error conditions</t>
   </si>
   <si>
+    <t>[EthFw][IPC]IPC: Integration with CPSW LLD RTOS driver running on A72/MCU_SS R5F remote core</t>
+  </si>
+  <si>
     <t>QRAS AP00216 Baseline Process</t>
   </si>
   <si>
     <t>Test Case Name</t>
   </si>
   <si>
+    <t>[EthFw][IPC]IPC: Support for remote core to query if switch R5 firmware has been loaded</t>
+  </si>
+  <si>
     <t>Version</t>
   </si>
   <si>
     <t>Execute cpsw baremetal test app and confirm successful execution</t>
   </si>
   <si>
+    <t>Ethernet Firmware IPC should be integrated with CPSW LLD RTOS driver running on MCU_SS R5F/C7x/C66x remote core</t>
+  </si>
+  <si>
     <t>Bug ID</t>
   </si>
   <si>
+    <t>EthFw switching app should run successfully on MCU_2_1 with TI RTOS configured in lock step mode</t>
+  </si>
+  <si>
+    <t>ETHFW-501</t>
+  </si>
+  <si>
     <t>EthFW EMAC OSAL Test - TI RTOS implementation</t>
   </si>
   <si>
@@ -539,21 +805,27 @@
     <t>[EthFW][OS]OSAL:EMAC Osal:Baremetal implementation of EMAL osal interface should be integrated into the switch firmware</t>
   </si>
   <si>
+    <t>ETHFW-51 : [EthFw][IPC]IPC: Support for remote core to query if switch R5 firmware has been loaded</t>
+  </si>
+  <si>
     <t>ETHFW-387</t>
   </si>
   <si>
     <t>Performance</t>
   </si>
   <si>
+    <t>ETHFW-495</t>
+  </si>
+  <si>
     <t>Customer Usage</t>
   </si>
   <si>
-    <t>7/18/2019</t>
-  </si>
-  <si>
     <t>Processor SDK Vision - EthFw</t>
   </si>
   <si>
+    <t>ETHSWITCHFW_J7_01.00.00_RTM</t>
+  </si>
+  <si>
     <t>Prasad Jondhale</t>
   </si>
   <si>
@@ -569,10 +841,10 @@
     <t>Downloaded from FoQus for 0.9 release and updated the summary tab and test details</t>
   </si>
   <si>
-    <t>EthFw_J7_00.09.00_BRINGUP</t>
-  </si>
-  <si>
-    <t>TI-RTOS</t>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Downloaded from FoQus for 1.0 release and updated the summary tab and test details</t>
   </si>
 </sst>
 </file>
@@ -1356,7 +1628,7 @@
     <xf numFmtId="9" fontId="12" fillId="2" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1548,22 +1820,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2063,12 +2323,12 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="57" t="s">
-        <v>166</v>
+        <v>252</v>
       </c>
       <c r="C2" s="58"/>
       <c r="D2" s="58"/>
@@ -2083,7 +2343,7 @@
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="63" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B4" s="64"/>
       <c r="C4" s="64"/>
@@ -2094,10 +2354,10 @@
     </row>
     <row r="5" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B5" s="66" t="s">
-        <v>172</v>
+        <v>259</v>
       </c>
       <c r="C5" s="67"/>
       <c r="D5" s="67"/>
@@ -2107,56 +2367,56 @@
     </row>
     <row r="6" spans="1:9" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B6" s="69" t="s">
-        <v>178</v>
-      </c>
-      <c r="C6" s="70"/>
-      <c r="D6" s="70"/>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="71"/>
+        <v>242</v>
+      </c>
+      <c r="B6" s="66" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="68"/>
     </row>
     <row r="7" spans="1:9" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="B7" s="66" t="s">
-        <v>171</v>
-      </c>
-      <c r="C7" s="72"/>
-      <c r="D7" s="72"/>
-      <c r="E7" s="72"/>
-      <c r="F7" s="72"/>
+        <v>38</v>
+      </c>
+      <c r="C7" s="67"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="67"/>
+      <c r="F7" s="67"/>
       <c r="G7" s="68"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
     </row>
     <row r="8" spans="1:9" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B8" s="66" t="s">
-        <v>141</v>
-      </c>
-      <c r="C8" s="72"/>
-      <c r="D8" s="72"/>
-      <c r="E8" s="72"/>
-      <c r="F8" s="72"/>
+        <v>214</v>
+      </c>
+      <c r="C8" s="67"/>
+      <c r="D8" s="67"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="67"/>
       <c r="G8" s="68"/>
     </row>
     <row r="9" spans="1:9" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B9" s="66" t="s">
-        <v>179</v>
-      </c>
-      <c r="C9" s="72"/>
-      <c r="D9" s="72"/>
-      <c r="E9" s="72"/>
-      <c r="F9" s="72"/>
+        <v>154</v>
+      </c>
+      <c r="C9" s="67"/>
+      <c r="D9" s="67"/>
+      <c r="E9" s="67"/>
+      <c r="F9" s="67"/>
       <c r="G9" s="68"/>
     </row>
     <row r="10" spans="1:9" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2165,7 +2425,7 @@
     <row r="11" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="12" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="60" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B12" s="61"/>
       <c r="C12" s="62"/>
@@ -2176,66 +2436,66 @@
     </row>
     <row r="13" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="B13" s="56" t="s">
-        <v>122</v>
+        <v>40</v>
       </c>
       <c r="C13" s="56"/>
     </row>
     <row r="14" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B14" s="9">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
-        <v>137</v>
+        <v>208</v>
       </c>
       <c r="B15" s="9">
         <v>0</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>165</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="B16" s="9">
         <v>0</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>165</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="B17" s="9">
         <v>0</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>165</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B18" s="9">
         <v>0</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>165</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -2251,14 +2511,14 @@
     <mergeCell ref="B9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE14"/>
+  <dimension ref="A1:AG31"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.42578125" style="1" customWidth="1"/>
@@ -2267,57 +2527,60 @@
     <col min="4" max="4" width="60.7109375" style="10" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" style="10" customWidth="1"/>
     <col min="6" max="6" width="34.42578125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="19.28515625" style="10" customWidth="1"/>
-    <col min="8" max="21" width="4.7109375" style="10" customWidth="1"/>
-    <col min="22" max="22" width="19.28515625" style="10" customWidth="1"/>
-    <col min="23" max="25" width="4.7109375" style="10" customWidth="1"/>
-    <col min="26" max="26" width="19.28515625" style="10" customWidth="1"/>
-    <col min="27" max="27" width="16.42578125" style="10" customWidth="1"/>
-    <col min="28" max="28" width="13.42578125" style="5" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="14.28515625" style="10" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="14.28515625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="30.42578125" style="10" customWidth="1"/>
+    <col min="8" max="9" width="19.28515625" style="10" customWidth="1"/>
+    <col min="10" max="23" width="4.7109375" style="10" customWidth="1"/>
+    <col min="24" max="24" width="19.28515625" style="10" customWidth="1"/>
+    <col min="25" max="27" width="4.7109375" style="10" customWidth="1"/>
+    <col min="28" max="28" width="19.28515625" style="10" customWidth="1"/>
+    <col min="29" max="29" width="16.42578125" style="10" customWidth="1"/>
+    <col min="30" max="30" width="13.42578125" style="5" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="14.28515625" style="10" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="14.28515625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:33" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>63</v>
-      </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="73"/>
-      <c r="Q2" s="73"/>
-      <c r="R2" s="73"/>
-      <c r="S2" s="73"/>
-      <c r="T2" s="73"/>
-      <c r="U2" s="73"/>
-      <c r="V2" s="73"/>
-      <c r="W2" s="73"/>
-      <c r="X2" s="73"/>
-      <c r="Y2" s="73"/>
-      <c r="Z2" s="73"/>
-      <c r="AA2" s="73"/>
-      <c r="AB2" s="73"/>
-      <c r="AC2" s="73"/>
-      <c r="AD2" s="73"/>
-    </row>
-    <row r="3" spans="1:31" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="69" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="69"/>
+      <c r="T2" s="69"/>
+      <c r="U2" s="69"/>
+      <c r="V2" s="69"/>
+      <c r="W2" s="69"/>
+      <c r="X2" s="69"/>
+      <c r="Y2" s="69"/>
+      <c r="Z2" s="69"/>
+      <c r="AA2" s="69"/>
+      <c r="AB2" s="69"/>
+      <c r="AC2" s="69"/>
+      <c r="AD2" s="69"/>
+      <c r="AE2" s="69"/>
+      <c r="AF2" s="69"/>
+    </row>
+    <row r="3" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -2347,9 +2610,11 @@
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
-      <c r="AD3" s="11"/>
-    </row>
-    <row r="4" spans="1:31" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="6"/>
+      <c r="AF3" s="11"/>
+    </row>
+    <row r="4" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -2357,564 +2622,1527 @@
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="74" t="s">
-        <v>98</v>
-      </c>
-      <c r="I4" s="75"/>
-      <c r="J4" s="75"/>
-      <c r="K4" s="75"/>
-      <c r="L4" s="75"/>
-      <c r="M4" s="75"/>
-      <c r="N4" s="76"/>
-      <c r="O4" s="74" t="s">
-        <v>139</v>
-      </c>
-      <c r="P4" s="75"/>
-      <c r="Q4" s="75"/>
-      <c r="R4" s="75"/>
-      <c r="S4" s="75"/>
-      <c r="T4" s="75"/>
-      <c r="U4" s="76"/>
-      <c r="V4" s="12"/>
-      <c r="W4" s="74" t="s">
-        <v>62</v>
-      </c>
-      <c r="X4" s="75"/>
-      <c r="Y4" s="76"/>
-      <c r="Z4" s="12"/>
-      <c r="AA4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="70" t="s">
+        <v>149</v>
+      </c>
+      <c r="K4" s="71"/>
+      <c r="L4" s="71"/>
+      <c r="M4" s="71"/>
+      <c r="N4" s="71"/>
+      <c r="O4" s="71"/>
+      <c r="P4" s="72"/>
+      <c r="Q4" s="70" t="s">
+        <v>210</v>
+      </c>
+      <c r="R4" s="71"/>
+      <c r="S4" s="71"/>
+      <c r="T4" s="71"/>
+      <c r="U4" s="71"/>
+      <c r="V4" s="71"/>
+      <c r="W4" s="72"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="70" t="s">
+        <v>93</v>
+      </c>
+      <c r="Z4" s="71"/>
+      <c r="AA4" s="72"/>
       <c r="AB4" s="12"/>
       <c r="AC4" s="12"/>
-      <c r="AD4" s="77" t="s">
-        <v>34</v>
-      </c>
-      <c r="AE4" s="78"/>
-    </row>
-    <row r="5" spans="1:31" s="13" customFormat="1" ht="86.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AD4" s="12"/>
+      <c r="AE4" s="12"/>
+      <c r="AF4" s="73" t="s">
+        <v>50</v>
+      </c>
+      <c r="AG4" s="74"/>
+    </row>
+    <row r="5" spans="1:33" s="13" customFormat="1" ht="86.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="L5" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="M5" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="N5" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="O5" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="P5" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q5" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="R5" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="S5" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="T5" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="U5" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="V5" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="W5" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="X5" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="Y5" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="AA5" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="AB5" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="AC5" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD5" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="AE5" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="H5" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="K5" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="L5" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="M5" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="N5" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="O5" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="P5" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q5" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="R5" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="S5" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="T5" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="U5" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="V5" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="W5" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="X5" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y5" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="Z5" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="AA5" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="AB5" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="AC5" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="AD5" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="AE5" s="16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:31" s="5" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="AF5" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="AG5" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" s="5" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
-        <v>90</v>
+        <v>137</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>163</v>
+        <v>249</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>1</v>
       </c>
       <c r="E6" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q6" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="X6" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA6" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB6" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC6" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF6" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG6" s="21" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>248</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="G7" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I7" s="23" t="s">
+        <v>223</v>
+      </c>
+      <c r="J7" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q7" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X7" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA7" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB7" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC7" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF7" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG7" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>250</v>
+      </c>
+      <c r="G8" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="J8" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q8" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X8" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA8" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB8" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC8" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF8" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG8" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A9" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="J9" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q9" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X9" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA9" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB9" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC9" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF9" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG9" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A10" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H10" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="J10" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q10" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X10" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA10" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB10" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC10" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF10" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG10" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" s="1" customFormat="1" ht="102" x14ac:dyDescent="0.2">
+      <c r="A11" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="J11" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q11" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X11" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA11" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB11" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC11" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF11" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG11" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:33" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="E12" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="G12" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="J12" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q12" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X12" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA12" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB12" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC12" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF12" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG12" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A13" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="G13" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="J13" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q13" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X13" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA13" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB13" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC13" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF13" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG13" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A14" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>255</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="E14" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="G14" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>226</v>
+      </c>
+      <c r="J14" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q14" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X14" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA14" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB14" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC14" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF14" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG14" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A15" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="G15" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I15" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="J15" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q15" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X15" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA15" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB15" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC15" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF15" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG15" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A16" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="G16" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>229</v>
+      </c>
+      <c r="J16" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q16" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X16" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA16" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB16" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC16" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF16" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG16" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:33" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A17" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I17" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="J17" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q17" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X17" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA17" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB17" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC17" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF17" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG17" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:33" s="1" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>220</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="G18" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H18" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I18" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="J18" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q18" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X18" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA18" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB18" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC18" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF18" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG18" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:33" s="1" customFormat="1" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="A19" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>241</v>
+      </c>
+      <c r="C19" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="D19" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="G19" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="J19" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q19" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X19" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA19" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB19" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC19" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF19" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG19" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="20" spans="1:33" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A20" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="E20" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="G20" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H20" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I20" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="J20" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q20" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X20" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA20" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB20" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC20" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF20" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG20" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="21" spans="1:33" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A21" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="B21" s="22" t="s">
+        <v>238</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>257</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="G21" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H21" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I21" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="J21" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q21" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X21" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA21" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB21" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC21" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF21" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG21" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="22" spans="1:33" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A22" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="G22" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H22" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I22" s="23" t="s">
+        <v>246</v>
+      </c>
+      <c r="J22" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q22" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X22" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA22" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB22" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC22" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF22" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG22" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="23" spans="1:33" s="1" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="C23" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="O6" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="V6" s="19" t="s">
+      <c r="D23" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="E23" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="G23" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H23" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I23" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="N23" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q23" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X23" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA23" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB23" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC23" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF23" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG23" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="24" spans="1:33" s="1" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G24" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H24" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I24" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="N24" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q24" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X24" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA24" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB24" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC24" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF24" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG24" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:33" s="1" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="G25" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H25" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="N25" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q25" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X25" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA25" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB25" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC25" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF25" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG25" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26" spans="1:33" s="1" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G26" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H26" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I26" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="N26" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q26" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X26" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA26" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB26" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC26" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF26" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG26" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:33" s="1" customFormat="1" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="A27" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>247</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="G27" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H27" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I27" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="N27" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q27" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X27" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA27" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB27" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC27" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF27" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG27" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:33" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A28" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="G28" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H28" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I28" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="N28" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q28" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X28" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA28" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB28" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC28" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF28" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG28" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="29" spans="1:33" s="1" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A29" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E29" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F29" s="23" t="s">
+        <v>177</v>
+      </c>
+      <c r="G29" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I29" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="N29" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q29" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X29" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA29" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB29" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC29" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF29" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG29" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:33" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A30" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E30" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F30" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="G30" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H30" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I30" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="N30" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q30" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X30" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA30" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB30" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC30" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF30" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG30" s="26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="31" spans="1:33" s="1" customFormat="1" ht="178.5" x14ac:dyDescent="0.2">
+      <c r="A31" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B31" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>185</v>
+      </c>
+      <c r="F31" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="Y6" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z6" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA6" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD6" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE6" s="21" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>162</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="H7" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="O7" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="V7" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y7" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z7" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA7" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD7" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE7" s="26" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" s="1" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A8" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>125</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>164</v>
-      </c>
-      <c r="G8" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="O8" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="V8" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y8" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z8" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA8" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD8" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE8" s="26" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="G9" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="H9" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="O9" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="V9" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y9" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z9" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA9" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD9" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE9" s="26" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" spans="1:31" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="E10" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="H10" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="O10" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="V10" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y10" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z10" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA10" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD10" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE10" s="26" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="11" spans="1:31" s="1" customFormat="1" ht="102" x14ac:dyDescent="0.2">
-      <c r="A11" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="C11" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="E11" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="G11" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="O11" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="V11" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y11" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z11" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA11" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE11" s="26" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" spans="1:31" s="1" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="E12" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="G12" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H12" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="O12" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="V12" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y12" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z12" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA12" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD12" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE12" s="26" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:31" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A13" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="E13" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="G13" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="H13" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="O13" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="V13" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y13" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z13" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA13" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD13" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE13" s="26" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="1:31" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A14" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="22" t="s">
-        <v>168</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="E14" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="H14" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="O14" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="V14" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y14" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z14" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA14" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD14" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE14" s="26" t="s">
-        <v>86</v>
+      <c r="G31" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="H31" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="I31" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="L31" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="U31" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="X31" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA31" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB31" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC31" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AF31" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG31" s="26" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A2:AD2"/>
-    <mergeCell ref="H4:N4"/>
-    <mergeCell ref="O4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="AD4:AE4"/>
+    <mergeCell ref="A2:AF2"/>
+    <mergeCell ref="J4:P4"/>
+    <mergeCell ref="Q4:W4"/>
+    <mergeCell ref="Y4:AA4"/>
+    <mergeCell ref="AF4:AG4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2935,18 +4163,18 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>77</v>
-      </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
+      <c r="A2" s="69" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
       <c r="I2" s="29"/>
@@ -2965,542 +4193,542 @@
     </row>
     <row r="4" spans="1:10" s="5" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="B4" s="33" t="s">
+        <v>157</v>
+      </c>
+      <c r="C4" s="92" t="s">
+        <v>199</v>
+      </c>
+      <c r="D4" s="93"/>
+      <c r="E4" s="34" t="s">
+        <v>239</v>
+      </c>
+      <c r="F4" s="34" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="91" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="83" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="84"/>
+      <c r="E5" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="F5" s="37" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="91"/>
+      <c r="B6" s="35" t="s">
+        <v>240</v>
+      </c>
+      <c r="C6" s="83" t="s">
+        <v>126</v>
+      </c>
+      <c r="D6" s="84"/>
+      <c r="E6" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="F6" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="91"/>
+      <c r="B7" s="35" t="s">
+        <v>205</v>
+      </c>
+      <c r="C7" s="83" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="84"/>
+      <c r="E7" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="91"/>
+      <c r="B8" s="40" t="s">
+        <v>140</v>
+      </c>
+      <c r="C8" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D8" s="86"/>
+      <c r="E8" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" s="1" customFormat="1" ht="53.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="91"/>
+      <c r="B9" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="85" t="s">
+        <v>230</v>
+      </c>
+      <c r="D9" s="86"/>
+      <c r="E9" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="F9" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="91"/>
+      <c r="B10" s="35" t="s">
+        <v>172</v>
+      </c>
+      <c r="C10" s="87" t="s">
+        <v>136</v>
+      </c>
+      <c r="D10" s="90"/>
+      <c r="E10" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="F10" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="91"/>
+      <c r="B11" s="35" t="s">
+        <v>222</v>
+      </c>
+      <c r="C11" s="87" t="s">
+        <v>215</v>
+      </c>
+      <c r="D11" s="88"/>
+      <c r="E11" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="41" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="91"/>
+      <c r="B12" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="C12" s="87" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" s="90"/>
+      <c r="E12" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="F12" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="91"/>
+      <c r="B13" s="40" t="s">
+        <v>202</v>
+      </c>
+      <c r="C13" s="87" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="90"/>
+      <c r="E13" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="F13" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="1" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="91"/>
+      <c r="B14" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="C14" s="81" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="82"/>
+      <c r="E14" s="104" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" s="107" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="91"/>
+      <c r="B15" s="79"/>
+      <c r="C15" s="42" t="s">
+        <v>207</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E15" s="105"/>
+      <c r="F15" s="108"/>
+    </row>
+    <row r="16" spans="1:10" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="91"/>
+      <c r="B16" s="79"/>
+      <c r="C16" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="105"/>
+      <c r="F16" s="108"/>
+    </row>
+    <row r="17" spans="1:6" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="91"/>
+      <c r="B17" s="79"/>
+      <c r="C17" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="105"/>
+      <c r="F17" s="108"/>
+    </row>
+    <row r="18" spans="1:6" s="1" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="91"/>
+      <c r="B18" s="79"/>
+      <c r="C18" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="E18" s="105"/>
+      <c r="F18" s="108"/>
+    </row>
+    <row r="19" spans="1:6" s="1" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="91"/>
+      <c r="B19" s="79"/>
+      <c r="C19" s="42" t="s">
+        <v>256</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="E19" s="105"/>
+      <c r="F19" s="108"/>
+    </row>
+    <row r="20" spans="1:6" s="1" customFormat="1" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="91"/>
+      <c r="B20" s="79"/>
+      <c r="C20" s="42" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>235</v>
+      </c>
+      <c r="E20" s="105"/>
+      <c r="F20" s="108"/>
+    </row>
+    <row r="21" spans="1:6" s="1" customFormat="1" ht="57.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="91"/>
+      <c r="B21" s="80"/>
+      <c r="C21" s="42" t="s">
+        <v>174</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="E21" s="106"/>
+      <c r="F21" s="109"/>
+    </row>
+    <row r="22" spans="1:6" s="1" customFormat="1" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="91"/>
+      <c r="B22" s="89" t="s">
+        <v>210</v>
+      </c>
+      <c r="C22" s="97" t="s">
         <v>103</v>
       </c>
-      <c r="C4" s="96" t="s">
+      <c r="D22" s="98"/>
+      <c r="E22" s="104" t="s">
+        <v>71</v>
+      </c>
+      <c r="F22" s="107" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="91"/>
+      <c r="B23" s="79"/>
+      <c r="C23" s="43" t="s">
+        <v>231</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="E23" s="105"/>
+      <c r="F23" s="108"/>
+    </row>
+    <row r="24" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="91"/>
+      <c r="B24" s="79"/>
+      <c r="C24" s="43" t="s">
+        <v>228</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="105"/>
+      <c r="F24" s="108"/>
+    </row>
+    <row r="25" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="91"/>
+      <c r="B25" s="79"/>
+      <c r="C25" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="E25" s="105"/>
+      <c r="F25" s="108"/>
+    </row>
+    <row r="26" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="91"/>
+      <c r="B26" s="79"/>
+      <c r="C26" s="43" t="s">
+        <v>234</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" s="105"/>
+      <c r="F26" s="108"/>
+    </row>
+    <row r="27" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="91"/>
+      <c r="B27" s="79"/>
+      <c r="C27" s="43" t="s">
+        <v>258</v>
+      </c>
+      <c r="D27" s="44" t="s">
+        <v>175</v>
+      </c>
+      <c r="E27" s="105"/>
+      <c r="F27" s="108"/>
+    </row>
+    <row r="28" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="91"/>
+      <c r="B28" s="79"/>
+      <c r="C28" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="44" t="s">
+        <v>237</v>
+      </c>
+      <c r="E28" s="105"/>
+      <c r="F28" s="108"/>
+    </row>
+    <row r="29" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="91"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="45" t="s">
+        <v>183</v>
+      </c>
+      <c r="D29" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="E29" s="106"/>
+      <c r="F29" s="109"/>
+    </row>
+    <row r="30" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="91"/>
+      <c r="B30" s="47" t="s">
+        <v>178</v>
+      </c>
+      <c r="C30" s="99" t="s">
+        <v>233</v>
+      </c>
+      <c r="D30" s="100"/>
+      <c r="E30" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="F30" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="91"/>
+      <c r="B31" s="75" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" s="87" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="90"/>
+      <c r="E31" s="104" t="s">
+        <v>71</v>
+      </c>
+      <c r="F31" s="107" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="91"/>
+      <c r="B32" s="76"/>
+      <c r="C32" s="48" t="s">
+        <v>28</v>
+      </c>
+      <c r="D32" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="E32" s="105"/>
+      <c r="F32" s="108"/>
+    </row>
+    <row r="33" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="91"/>
+      <c r="B33" s="76"/>
+      <c r="C33" s="48" t="s">
+        <v>82</v>
+      </c>
+      <c r="D33" s="50" t="s">
+        <v>227</v>
+      </c>
+      <c r="E33" s="105"/>
+      <c r="F33" s="108"/>
+    </row>
+    <row r="34" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="91"/>
+      <c r="B34" s="77"/>
+      <c r="C34" s="48" t="s">
+        <v>145</v>
+      </c>
+      <c r="D34" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="E34" s="106"/>
+      <c r="F34" s="109"/>
+    </row>
+    <row r="35" spans="1:6" s="1" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="94" t="s">
+        <v>112</v>
+      </c>
+      <c r="B35" s="35" t="s">
+        <v>142</v>
+      </c>
+      <c r="C35" s="87" t="s">
         <v>129</v>
       </c>
-      <c r="D4" s="97"/>
-      <c r="E4" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="F4" s="34" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="95" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="87" t="s">
-        <v>95</v>
-      </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="36" t="s">
-        <v>133</v>
-      </c>
-      <c r="F5" s="37" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="95"/>
-      <c r="B6" s="35" t="s">
-        <v>158</v>
-      </c>
-      <c r="C6" s="87" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F6" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="95"/>
-      <c r="B7" s="35" t="s">
-        <v>134</v>
-      </c>
-      <c r="C7" s="87" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="88"/>
-      <c r="E7" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F7" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="95"/>
-      <c r="B8" s="40" t="s">
-        <v>92</v>
-      </c>
-      <c r="C8" s="89" t="s">
-        <v>143</v>
-      </c>
-      <c r="D8" s="90"/>
-      <c r="E8" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F8" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="53.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="95"/>
-      <c r="B9" s="40" t="s">
+      <c r="D35" s="90"/>
+      <c r="E35" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="F35" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="94"/>
+      <c r="B36" s="35" t="s">
+        <v>245</v>
+      </c>
+      <c r="C36" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="89" t="s">
-        <v>149</v>
-      </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="41" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="95"/>
-      <c r="B10" s="35" t="s">
-        <v>114</v>
-      </c>
-      <c r="C10" s="91" t="s">
-        <v>89</v>
-      </c>
-      <c r="D10" s="94"/>
-      <c r="E10" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F10" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="95"/>
-      <c r="B11" s="35" t="s">
-        <v>144</v>
-      </c>
-      <c r="C11" s="91" t="s">
-        <v>142</v>
-      </c>
-      <c r="D11" s="92"/>
-      <c r="E11" s="41" t="s">
-        <v>49</v>
-      </c>
-      <c r="F11" s="41" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="95"/>
-      <c r="B12" s="35" t="s">
-        <v>126</v>
-      </c>
-      <c r="C12" s="91" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="94"/>
-      <c r="E12" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F12" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="95"/>
-      <c r="B13" s="40" t="s">
-        <v>131</v>
-      </c>
-      <c r="C13" s="91" t="s">
+      <c r="D36" s="90"/>
+      <c r="E36" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="F36" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="94"/>
+      <c r="B37" s="75" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" s="95" t="s">
+        <v>181</v>
+      </c>
+      <c r="D37" s="96"/>
+      <c r="E37" s="101" t="s">
+        <v>204</v>
+      </c>
+      <c r="F37" s="107" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="94"/>
+      <c r="B38" s="76"/>
+      <c r="C38" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="44" t="s">
+        <v>70</v>
+      </c>
+      <c r="E38" s="102"/>
+      <c r="F38" s="108"/>
+    </row>
+    <row r="39" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="94"/>
+      <c r="B39" s="76"/>
+      <c r="C39" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="94"/>
-      <c r="E13" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F13" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" s="1" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="95"/>
-      <c r="B14" s="82" t="s">
-        <v>98</v>
-      </c>
-      <c r="C14" s="85" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="86"/>
-      <c r="E14" s="108" t="s">
-        <v>49</v>
-      </c>
-      <c r="F14" s="111" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="95"/>
-      <c r="B15" s="83"/>
-      <c r="C15" s="42" t="s">
-        <v>136</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="E15" s="109"/>
-      <c r="F15" s="112"/>
-    </row>
-    <row r="16" spans="1:10" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="95"/>
-      <c r="B16" s="83"/>
-      <c r="C16" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="23" t="s">
+      <c r="D39" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E39" s="102"/>
+      <c r="F39" s="108"/>
+    </row>
+    <row r="40" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="94"/>
+      <c r="B40" s="76"/>
+      <c r="C40" s="43" t="s">
+        <v>208</v>
+      </c>
+      <c r="D40" s="44" t="s">
+        <v>147</v>
+      </c>
+      <c r="E40" s="102"/>
+      <c r="F40" s="108"/>
+    </row>
+    <row r="41" spans="1:6" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A41" s="94"/>
+      <c r="B41" s="76"/>
+      <c r="C41" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="109"/>
-      <c r="F16" s="112"/>
-    </row>
-    <row r="17" spans="1:6" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="95"/>
-      <c r="B17" s="83"/>
-      <c r="C17" s="42" t="s">
-        <v>109</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" s="109"/>
-      <c r="F17" s="112"/>
-    </row>
-    <row r="18" spans="1:6" s="1" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="95"/>
-      <c r="B18" s="83"/>
-      <c r="C18" s="42" t="s">
-        <v>87</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>110</v>
-      </c>
-      <c r="E18" s="109"/>
-      <c r="F18" s="112"/>
-    </row>
-    <row r="19" spans="1:6" s="1" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="95"/>
-      <c r="B19" s="83"/>
-      <c r="C19" s="42" t="s">
-        <v>169</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="E19" s="109"/>
-      <c r="F19" s="112"/>
-    </row>
-    <row r="20" spans="1:6" s="1" customFormat="1" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="95"/>
-      <c r="B20" s="83"/>
-      <c r="C20" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="E20" s="109"/>
-      <c r="F20" s="112"/>
-    </row>
-    <row r="21" spans="1:6" s="1" customFormat="1" ht="57.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="95"/>
-      <c r="B21" s="84"/>
-      <c r="C21" s="42" t="s">
-        <v>115</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="E21" s="110"/>
-      <c r="F21" s="113"/>
-    </row>
-    <row r="22" spans="1:6" s="1" customFormat="1" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="95"/>
-      <c r="B22" s="93" t="s">
-        <v>139</v>
-      </c>
-      <c r="C22" s="101" t="s">
-        <v>70</v>
-      </c>
-      <c r="D22" s="102"/>
-      <c r="E22" s="108" t="s">
-        <v>49</v>
-      </c>
-      <c r="F22" s="111" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="95"/>
-      <c r="B23" s="83"/>
-      <c r="C23" s="43" t="s">
-        <v>150</v>
-      </c>
-      <c r="D23" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="E23" s="109"/>
-      <c r="F23" s="112"/>
-    </row>
-    <row r="24" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="95"/>
-      <c r="B24" s="83"/>
-      <c r="C24" s="43" t="s">
-        <v>148</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="E24" s="109"/>
-      <c r="F24" s="112"/>
-    </row>
-    <row r="25" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="95"/>
-      <c r="B25" s="83"/>
-      <c r="C25" s="43" t="s">
-        <v>113</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="E25" s="109"/>
-      <c r="F25" s="112"/>
-    </row>
-    <row r="26" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="95"/>
-      <c r="B26" s="83"/>
-      <c r="C26" s="43" t="s">
-        <v>152</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" s="109"/>
-      <c r="F26" s="112"/>
-    </row>
-    <row r="27" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="95"/>
-      <c r="B27" s="83"/>
-      <c r="C27" s="43" t="s">
-        <v>170</v>
-      </c>
-      <c r="D27" s="44" t="s">
-        <v>116</v>
-      </c>
-      <c r="E27" s="109"/>
-      <c r="F27" s="112"/>
-    </row>
-    <row r="28" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="95"/>
-      <c r="B28" s="83"/>
-      <c r="C28" s="43" t="s">
-        <v>41</v>
-      </c>
-      <c r="D28" s="44" t="s">
-        <v>156</v>
-      </c>
-      <c r="E28" s="109"/>
-      <c r="F28" s="112"/>
-    </row>
-    <row r="29" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="95"/>
-      <c r="B29" s="84"/>
-      <c r="C29" s="45" t="s">
-        <v>121</v>
-      </c>
-      <c r="D29" s="46" t="s">
-        <v>106</v>
-      </c>
-      <c r="E29" s="110"/>
-      <c r="F29" s="113"/>
-    </row>
-    <row r="30" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="95"/>
-      <c r="B30" s="47" t="s">
-        <v>117</v>
-      </c>
-      <c r="C30" s="103" t="s">
-        <v>151</v>
-      </c>
-      <c r="D30" s="104"/>
-      <c r="E30" s="41" t="s">
-        <v>49</v>
-      </c>
-      <c r="F30" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="95"/>
-      <c r="B31" s="79" t="s">
-        <v>62</v>
-      </c>
-      <c r="C31" s="91" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="94"/>
-      <c r="E31" s="108" t="s">
-        <v>49</v>
-      </c>
-      <c r="F31" s="111" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="95"/>
-      <c r="B32" s="80"/>
-      <c r="C32" s="48" t="s">
-        <v>18</v>
-      </c>
-      <c r="D32" s="49" t="s">
-        <v>17</v>
-      </c>
-      <c r="E32" s="109"/>
-      <c r="F32" s="112"/>
-    </row>
-    <row r="33" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="95"/>
-      <c r="B33" s="80"/>
-      <c r="C33" s="48" t="s">
-        <v>56</v>
-      </c>
-      <c r="D33" s="50" t="s">
-        <v>147</v>
-      </c>
-      <c r="E33" s="109"/>
-      <c r="F33" s="112"/>
-    </row>
-    <row r="34" spans="1:6" s="1" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="95"/>
-      <c r="B34" s="81"/>
-      <c r="C34" s="48" t="s">
-        <v>94</v>
-      </c>
-      <c r="D34" s="50" t="s">
-        <v>64</v>
-      </c>
-      <c r="E34" s="110"/>
-      <c r="F34" s="113"/>
-    </row>
-    <row r="35" spans="1:6" s="1" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="98" t="s">
-        <v>76</v>
-      </c>
-      <c r="B35" s="35" t="s">
-        <v>93</v>
-      </c>
-      <c r="C35" s="91" t="s">
-        <v>84</v>
-      </c>
-      <c r="D35" s="94"/>
-      <c r="E35" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F35" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="98"/>
-      <c r="B36" s="35" t="s">
-        <v>161</v>
-      </c>
-      <c r="C36" s="91" t="s">
-        <v>38</v>
-      </c>
-      <c r="D36" s="94"/>
-      <c r="E36" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F36" s="39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="98"/>
-      <c r="B37" s="79" t="s">
-        <v>34</v>
-      </c>
-      <c r="C37" s="99" t="s">
-        <v>119</v>
-      </c>
-      <c r="D37" s="100"/>
-      <c r="E37" s="105" t="s">
-        <v>133</v>
-      </c>
-      <c r="F37" s="111" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="98"/>
-      <c r="B38" s="80"/>
-      <c r="C38" s="43" t="s">
-        <v>11</v>
-      </c>
-      <c r="D38" s="44" t="s">
-        <v>48</v>
-      </c>
-      <c r="E38" s="106"/>
-      <c r="F38" s="112"/>
-    </row>
-    <row r="39" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="98"/>
-      <c r="B39" s="80"/>
-      <c r="C39" s="43" t="s">
-        <v>9</v>
-      </c>
-      <c r="D39" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="E39" s="106"/>
-      <c r="F39" s="112"/>
-    </row>
-    <row r="40" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="98"/>
-      <c r="B40" s="80"/>
-      <c r="C40" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="D40" s="44" t="s">
-        <v>96</v>
-      </c>
-      <c r="E40" s="106"/>
-      <c r="F40" s="112"/>
-    </row>
-    <row r="41" spans="1:6" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A41" s="98"/>
-      <c r="B41" s="80"/>
-      <c r="C41" s="43" t="s">
-        <v>37</v>
-      </c>
       <c r="D41" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="E41" s="106"/>
-      <c r="F41" s="112"/>
+        <v>57</v>
+      </c>
+      <c r="E41" s="102"/>
+      <c r="F41" s="108"/>
     </row>
     <row r="42" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="98"/>
-      <c r="B42" s="81"/>
+      <c r="A42" s="94"/>
+      <c r="B42" s="77"/>
       <c r="C42" s="51" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="D42" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E42" s="107"/>
-      <c r="F42" s="114"/>
+      <c r="E42" s="103"/>
+      <c r="F42" s="110"/>
     </row>
   </sheetData>
   <mergeCells count="32">
@@ -3544,7 +4772,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.7109375" style="1" customWidth="1"/>
@@ -3555,41 +4783,41 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="115" t="s">
-        <v>65</v>
-      </c>
-      <c r="B3" s="115"/>
-      <c r="C3" s="115"/>
-      <c r="D3" s="116"/>
+      <c r="A3" s="111" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="111"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="112"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="117"/>
-      <c r="B4" s="117"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="118"/>
+      <c r="A4" s="113"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="113"/>
+      <c r="D4" s="114"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="119"/>
-      <c r="B5" s="119"/>
-      <c r="C5" s="119"/>
-      <c r="D5" s="120"/>
+      <c r="A5" s="115"/>
+      <c r="B5" s="115"/>
+      <c r="C5" s="115"/>
+      <c r="D5" s="116"/>
     </row>
     <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A6" s="52" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B6" s="52" t="s">
-        <v>159</v>
+        <v>242</v>
       </c>
       <c r="C6" s="52" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="D6" s="52" t="s">
-        <v>129</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -3617,107 +4845,121 @@
       <c r="D10" s="53"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="115" t="s">
-        <v>124</v>
-      </c>
-      <c r="B15" s="115"/>
-      <c r="C15" s="115"/>
-      <c r="D15" s="116"/>
+      <c r="A15" s="111" t="s">
+        <v>191</v>
+      </c>
+      <c r="B15" s="111"/>
+      <c r="C15" s="111"/>
+      <c r="D15" s="112"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="117"/>
-      <c r="B16" s="117"/>
-      <c r="C16" s="117"/>
-      <c r="D16" s="118"/>
+      <c r="A16" s="113"/>
+      <c r="B16" s="113"/>
+      <c r="C16" s="113"/>
+      <c r="D16" s="114"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="119"/>
-      <c r="B17" s="119"/>
-      <c r="C17" s="119"/>
-      <c r="D17" s="120"/>
+      <c r="A17" s="115"/>
+      <c r="B17" s="115"/>
+      <c r="C17" s="115"/>
+      <c r="D17" s="116"/>
     </row>
     <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A18" s="52" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>159</v>
+        <v>242</v>
       </c>
       <c r="C18" s="52" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="D18" s="52" t="s">
-        <v>129</v>
+        <v>199</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="53" t="s">
-        <v>130</v>
+        <v>201</v>
       </c>
       <c r="B19" s="54" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C19" s="55">
         <v>43343</v>
       </c>
       <c r="D19" s="53" t="s">
-        <v>111</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A20" s="53" t="s">
-        <v>130</v>
+        <v>201</v>
       </c>
       <c r="B20" s="54" t="s">
-        <v>102</v>
+        <v>155</v>
       </c>
       <c r="C20" s="55">
         <v>43396</v>
       </c>
       <c r="D20" s="53" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A21" s="53" t="s">
-        <v>130</v>
+        <v>201</v>
       </c>
       <c r="B21" s="54" t="s">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="C21" s="55">
         <v>43413</v>
       </c>
       <c r="D21" s="53" t="s">
-        <v>81</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A22" s="53" t="s">
-        <v>173</v>
+        <v>261</v>
       </c>
       <c r="B22" s="54" t="s">
-        <v>174</v>
+        <v>262</v>
       </c>
       <c r="C22" s="55">
         <v>43558</v>
       </c>
       <c r="D22" s="53" t="s">
-        <v>175</v>
+        <v>263</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A23" s="53" t="s">
-        <v>173</v>
+        <v>261</v>
       </c>
       <c r="B23" s="54" t="s">
-        <v>176</v>
+        <v>264</v>
       </c>
       <c r="C23" s="55">
         <v>43664</v>
       </c>
       <c r="D23" s="53" t="s">
-        <v>177</v>
+        <v>265</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A24" s="53" t="s">
+        <v>261</v>
+      </c>
+      <c r="B24" s="54" t="s">
+        <v>266</v>
+      </c>
+      <c r="C24" s="55">
+        <v>43756</v>
+      </c>
+      <c r="D24" s="53" t="s">
+        <v>267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>